<commit_message>
updated planning, update component's choice, electronics design
</commit_message>
<xml_diff>
--- a/A_Documentation/Planning.xlsx
+++ b/A_Documentation/Planning.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6270b752bd77e45c/Travail/HEIG-VD/Semestre_6/TB_2026/A_Documentation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\Documents\Repositories\Self-Balancing-Bot\A_Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="267" documentId="13_ncr:1_{EB2344AB-5E35-4500-9417-5A6D8235FE5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA20CBF7-0407-497B-AB3A-3A53B4B402A2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ADB7339-9F1C-4CD5-AFEF-27F344788BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -625,7 +625,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -781,6 +781,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2083,15 +2084,15 @@
       <c r="R16" s="7"/>
       <c r="S16" s="7"/>
       <c r="T16" s="7"/>
-      <c r="U16" s="7"/>
-      <c r="V16" s="7"/>
-      <c r="W16" s="7"/>
+      <c r="U16" s="10"/>
+      <c r="V16" s="10"/>
+      <c r="W16" s="10"/>
       <c r="X16" s="7"/>
-      <c r="Y16" s="7"/>
-      <c r="Z16" s="7"/>
-      <c r="AA16" s="7"/>
-      <c r="AB16" s="7"/>
-      <c r="AC16" s="7"/>
+      <c r="Y16" s="10"/>
+      <c r="Z16" s="67"/>
+      <c r="AA16" s="67"/>
+      <c r="AB16" s="67"/>
+      <c r="AC16" s="67"/>
       <c r="AD16" s="7"/>
       <c r="AE16" s="7"/>
       <c r="AF16" s="7"/>
@@ -2335,20 +2336,20 @@
       <c r="N20" s="7"/>
       <c r="O20" s="7"/>
       <c r="P20" s="10"/>
-      <c r="Q20" s="7"/>
-      <c r="R20" s="7"/>
-      <c r="S20" s="7"/>
-      <c r="T20" s="7"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="10"/>
+      <c r="S20" s="10"/>
+      <c r="T20" s="10"/>
       <c r="U20" s="7"/>
       <c r="V20" s="7"/>
-      <c r="W20" s="7"/>
-      <c r="X20" s="7"/>
-      <c r="Y20" s="7"/>
-      <c r="Z20" s="7"/>
-      <c r="AA20" s="7"/>
-      <c r="AB20" s="7"/>
-      <c r="AC20" s="7"/>
-      <c r="AD20" s="7"/>
+      <c r="W20" s="10"/>
+      <c r="X20" s="10"/>
+      <c r="Y20" s="10"/>
+      <c r="Z20" s="67"/>
+      <c r="AA20" s="67"/>
+      <c r="AB20" s="67"/>
+      <c r="AC20" s="67"/>
+      <c r="AD20" s="67"/>
       <c r="AE20" s="7"/>
       <c r="AF20" s="7"/>
       <c r="AG20" s="7"/>

</xml_diff>

<commit_message>
Modified Battery support (Added groove), Modified fall protection, TPU
</commit_message>
<xml_diff>
--- a/A_Documentation/Planning.xlsx
+++ b/A_Documentation/Planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\Documents\Repositories\Self-Balancing-Bot\A_Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ADB7339-9F1C-4CD5-AFEF-27F344788BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13006F8B-8917-450D-B57A-9B2B7D63ACDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -625,7 +625,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -667,6 +667,51 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -685,50 +730,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -738,24 +747,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -781,7 +772,15 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1209,12 +1208,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="47"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -1222,29 +1221,29 @@
       <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="48" t="s">
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="49"/>
+      <c r="G2" s="32"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="48" t="s">
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="49"/>
+      <c r="G3" s="32"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:61" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -1252,165 +1251,165 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="42" t="s">
+      <c r="F4" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="43"/>
+      <c r="G4" s="34"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="44">
         <v>25</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="31"/>
-      <c r="L5" s="29">
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="46"/>
+      <c r="L5" s="44">
         <v>26</v>
       </c>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
-      <c r="P5" s="30"/>
-      <c r="Q5" s="30"/>
-      <c r="R5" s="30"/>
-      <c r="S5" s="30"/>
-      <c r="T5" s="30"/>
-      <c r="U5" s="31"/>
-      <c r="V5" s="29">
+      <c r="M5" s="45"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="45"/>
+      <c r="P5" s="45"/>
+      <c r="Q5" s="45"/>
+      <c r="R5" s="45"/>
+      <c r="S5" s="45"/>
+      <c r="T5" s="45"/>
+      <c r="U5" s="46"/>
+      <c r="V5" s="44">
         <v>27</v>
       </c>
-      <c r="W5" s="30"/>
-      <c r="X5" s="30"/>
-      <c r="Y5" s="30"/>
-      <c r="Z5" s="30"/>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="30"/>
-      <c r="AC5" s="30"/>
-      <c r="AD5" s="30"/>
-      <c r="AE5" s="31"/>
-      <c r="AF5" s="29">
+      <c r="W5" s="45"/>
+      <c r="X5" s="45"/>
+      <c r="Y5" s="45"/>
+      <c r="Z5" s="45"/>
+      <c r="AA5" s="45"/>
+      <c r="AB5" s="45"/>
+      <c r="AC5" s="45"/>
+      <c r="AD5" s="45"/>
+      <c r="AE5" s="46"/>
+      <c r="AF5" s="44">
         <v>28</v>
       </c>
-      <c r="AG5" s="30"/>
-      <c r="AH5" s="30"/>
-      <c r="AI5" s="30"/>
-      <c r="AJ5" s="30"/>
-      <c r="AK5" s="30"/>
-      <c r="AL5" s="30"/>
-      <c r="AM5" s="30"/>
-      <c r="AN5" s="30"/>
-      <c r="AO5" s="31"/>
-      <c r="AP5" s="29">
+      <c r="AG5" s="45"/>
+      <c r="AH5" s="45"/>
+      <c r="AI5" s="45"/>
+      <c r="AJ5" s="45"/>
+      <c r="AK5" s="45"/>
+      <c r="AL5" s="45"/>
+      <c r="AM5" s="45"/>
+      <c r="AN5" s="45"/>
+      <c r="AO5" s="46"/>
+      <c r="AP5" s="44">
         <v>29</v>
       </c>
-      <c r="AQ5" s="30"/>
-      <c r="AR5" s="30"/>
-      <c r="AS5" s="30"/>
-      <c r="AT5" s="30"/>
-      <c r="AU5" s="30"/>
-      <c r="AV5" s="30"/>
-      <c r="AW5" s="30"/>
-      <c r="AX5" s="30"/>
-      <c r="AY5" s="31"/>
-      <c r="AZ5" s="29">
+      <c r="AQ5" s="45"/>
+      <c r="AR5" s="45"/>
+      <c r="AS5" s="45"/>
+      <c r="AT5" s="45"/>
+      <c r="AU5" s="45"/>
+      <c r="AV5" s="45"/>
+      <c r="AW5" s="45"/>
+      <c r="AX5" s="45"/>
+      <c r="AY5" s="46"/>
+      <c r="AZ5" s="44">
         <v>30</v>
       </c>
-      <c r="BA5" s="30"/>
-      <c r="BB5" s="30"/>
-      <c r="BC5" s="30"/>
-      <c r="BD5" s="30"/>
-      <c r="BE5" s="30"/>
-      <c r="BF5" s="30"/>
-      <c r="BG5" s="30"/>
-      <c r="BH5" s="30"/>
-      <c r="BI5" s="31"/>
+      <c r="BA5" s="45"/>
+      <c r="BB5" s="45"/>
+      <c r="BC5" s="45"/>
+      <c r="BD5" s="45"/>
+      <c r="BE5" s="45"/>
+      <c r="BF5" s="45"/>
+      <c r="BG5" s="45"/>
+      <c r="BH5" s="45"/>
+      <c r="BI5" s="46"/>
     </row>
     <row r="6" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="33"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="32" t="s">
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="33"/>
-      <c r="N6" s="33"/>
-      <c r="O6" s="33"/>
-      <c r="P6" s="33"/>
-      <c r="Q6" s="33"/>
-      <c r="R6" s="33"/>
-      <c r="S6" s="33"/>
-      <c r="T6" s="33"/>
-      <c r="U6" s="34"/>
-      <c r="V6" s="32" t="s">
+      <c r="M6" s="48"/>
+      <c r="N6" s="48"/>
+      <c r="O6" s="48"/>
+      <c r="P6" s="48"/>
+      <c r="Q6" s="48"/>
+      <c r="R6" s="48"/>
+      <c r="S6" s="48"/>
+      <c r="T6" s="48"/>
+      <c r="U6" s="49"/>
+      <c r="V6" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="W6" s="33"/>
-      <c r="X6" s="33"/>
-      <c r="Y6" s="33"/>
-      <c r="Z6" s="33"/>
-      <c r="AA6" s="33"/>
-      <c r="AB6" s="33"/>
-      <c r="AC6" s="33"/>
-      <c r="AD6" s="33"/>
-      <c r="AE6" s="34"/>
-      <c r="AF6" s="32" t="s">
+      <c r="W6" s="48"/>
+      <c r="X6" s="48"/>
+      <c r="Y6" s="48"/>
+      <c r="Z6" s="48"/>
+      <c r="AA6" s="48"/>
+      <c r="AB6" s="48"/>
+      <c r="AC6" s="48"/>
+      <c r="AD6" s="48"/>
+      <c r="AE6" s="49"/>
+      <c r="AF6" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="AG6" s="33"/>
-      <c r="AH6" s="33"/>
-      <c r="AI6" s="33"/>
-      <c r="AJ6" s="33"/>
-      <c r="AK6" s="33"/>
-      <c r="AL6" s="33"/>
-      <c r="AM6" s="33"/>
-      <c r="AN6" s="33"/>
-      <c r="AO6" s="34"/>
-      <c r="AP6" s="32" t="s">
+      <c r="AG6" s="48"/>
+      <c r="AH6" s="48"/>
+      <c r="AI6" s="48"/>
+      <c r="AJ6" s="48"/>
+      <c r="AK6" s="48"/>
+      <c r="AL6" s="48"/>
+      <c r="AM6" s="48"/>
+      <c r="AN6" s="48"/>
+      <c r="AO6" s="49"/>
+      <c r="AP6" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="AQ6" s="33"/>
-      <c r="AR6" s="33"/>
-      <c r="AS6" s="33"/>
-      <c r="AT6" s="33"/>
-      <c r="AU6" s="33"/>
-      <c r="AV6" s="33"/>
-      <c r="AW6" s="33"/>
-      <c r="AX6" s="33"/>
-      <c r="AY6" s="34"/>
-      <c r="AZ6" s="32" t="s">
+      <c r="AQ6" s="48"/>
+      <c r="AR6" s="48"/>
+      <c r="AS6" s="48"/>
+      <c r="AT6" s="48"/>
+      <c r="AU6" s="48"/>
+      <c r="AV6" s="48"/>
+      <c r="AW6" s="48"/>
+      <c r="AX6" s="48"/>
+      <c r="AY6" s="49"/>
+      <c r="AZ6" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="BA6" s="33"/>
-      <c r="BB6" s="33"/>
-      <c r="BC6" s="33"/>
-      <c r="BD6" s="33"/>
-      <c r="BE6" s="33"/>
-      <c r="BF6" s="33"/>
-      <c r="BG6" s="33"/>
-      <c r="BH6" s="33"/>
-      <c r="BI6" s="34"/>
+      <c r="BA6" s="48"/>
+      <c r="BB6" s="48"/>
+      <c r="BC6" s="48"/>
+      <c r="BD6" s="48"/>
+      <c r="BE6" s="48"/>
+      <c r="BF6" s="48"/>
+      <c r="BG6" s="48"/>
+      <c r="BH6" s="48"/>
+      <c r="BI6" s="49"/>
     </row>
     <row r="7" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -1601,18 +1600,18 @@
       <c r="A8" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="AZ8" s="39" t="s">
+      <c r="AZ8" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="BA8" s="40"/>
-      <c r="BB8" s="40"/>
-      <c r="BC8" s="40"/>
-      <c r="BD8" s="40"/>
-      <c r="BE8" s="40"/>
-      <c r="BF8" s="40"/>
-      <c r="BG8" s="40"/>
-      <c r="BH8" s="40"/>
-      <c r="BI8" s="41"/>
+      <c r="BA8" s="42"/>
+      <c r="BB8" s="42"/>
+      <c r="BC8" s="42"/>
+      <c r="BD8" s="42"/>
+      <c r="BE8" s="42"/>
+      <c r="BF8" s="42"/>
+      <c r="BG8" s="42"/>
+      <c r="BH8" s="42"/>
+      <c r="BI8" s="43"/>
     </row>
     <row r="9" spans="1:61" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -1961,7 +1960,7 @@
       <c r="W14" s="7"/>
       <c r="X14" s="7"/>
       <c r="Y14" s="7"/>
-      <c r="Z14" s="7"/>
+      <c r="Z14" s="10"/>
       <c r="AA14" s="7"/>
       <c r="AB14" s="7"/>
       <c r="AC14" s="7"/>
@@ -2089,10 +2088,10 @@
       <c r="W16" s="10"/>
       <c r="X16" s="7"/>
       <c r="Y16" s="10"/>
-      <c r="Z16" s="67"/>
-      <c r="AA16" s="67"/>
-      <c r="AB16" s="67"/>
-      <c r="AC16" s="67"/>
+      <c r="Z16" s="7"/>
+      <c r="AA16" s="7"/>
+      <c r="AB16" s="7"/>
+      <c r="AC16" s="7"/>
       <c r="AD16" s="7"/>
       <c r="AE16" s="7"/>
       <c r="AF16" s="7"/>
@@ -2345,11 +2344,11 @@
       <c r="W20" s="10"/>
       <c r="X20" s="10"/>
       <c r="Y20" s="10"/>
-      <c r="Z20" s="67"/>
-      <c r="AA20" s="67"/>
-      <c r="AB20" s="67"/>
-      <c r="AC20" s="67"/>
-      <c r="AD20" s="67"/>
+      <c r="Z20" s="10"/>
+      <c r="AA20" s="7"/>
+      <c r="AB20" s="7"/>
+      <c r="AC20" s="7"/>
+      <c r="AD20" s="7"/>
       <c r="AE20" s="7"/>
       <c r="AF20" s="7"/>
       <c r="AG20" s="7"/>
@@ -3277,7 +3276,7 @@
       <c r="BI34" s="7"/>
     </row>
     <row r="35" spans="1:61" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="44" t="s">
+      <c r="A35" s="39" t="s">
         <v>40</v>
       </c>
       <c r="B35" s="5"/>
@@ -3342,7 +3341,7 @@
       <c r="BI35" s="24"/>
     </row>
     <row r="36" spans="1:61" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="45"/>
+      <c r="A36" s="40"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
@@ -5550,11 +5549,35 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="AZ6:BI6"/>
+    <mergeCell ref="L5:U5"/>
+    <mergeCell ref="V5:AE5"/>
+    <mergeCell ref="AF5:AO5"/>
+    <mergeCell ref="AP5:AY5"/>
+    <mergeCell ref="AZ5:BI5"/>
+    <mergeCell ref="B6:K6"/>
+    <mergeCell ref="L6:U6"/>
+    <mergeCell ref="V6:AE6"/>
+    <mergeCell ref="AF6:AO6"/>
+    <mergeCell ref="AP6:AY6"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="AZ8:BI8"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A61:A62"/>
     <mergeCell ref="A63:A64"/>
@@ -5571,35 +5594,11 @@
     <mergeCell ref="A33:A34"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="AZ8:BI8"/>
-    <mergeCell ref="B5:K5"/>
-    <mergeCell ref="AZ6:BI6"/>
-    <mergeCell ref="L5:U5"/>
-    <mergeCell ref="V5:AE5"/>
-    <mergeCell ref="AF5:AO5"/>
-    <mergeCell ref="AP5:AY5"/>
-    <mergeCell ref="AZ5:BI5"/>
-    <mergeCell ref="B6:K6"/>
-    <mergeCell ref="L6:U6"/>
-    <mergeCell ref="V6:AE6"/>
-    <mergeCell ref="AF6:AO6"/>
-    <mergeCell ref="AP6:AY6"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5619,12 +5618,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="47"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -5643,29 +5642,29 @@
       <c r="Q1" s="17"/>
     </row>
     <row r="2" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="48" t="s">
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="49"/>
+      <c r="G2" s="32"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="48" t="s">
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="49"/>
+      <c r="G3" s="32"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:52" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -5673,222 +5672,222 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="42" t="s">
+      <c r="F4" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="43"/>
+      <c r="G4" s="34"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="44">
         <v>8</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="29">
+      <c r="C5" s="45"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="44">
         <v>9</v>
       </c>
-      <c r="F5" s="30"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="50" t="s">
+      <c r="F5" s="45"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="51"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="29">
+      <c r="I5" s="54"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="44">
         <v>11</v>
       </c>
-      <c r="L5" s="30"/>
-      <c r="M5" s="31"/>
-      <c r="N5" s="50" t="s">
+      <c r="L5" s="45"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="51"/>
-      <c r="P5" s="52"/>
-      <c r="Q5" s="29">
+      <c r="O5" s="54"/>
+      <c r="P5" s="55"/>
+      <c r="Q5" s="44">
         <v>13</v>
       </c>
-      <c r="R5" s="30"/>
-      <c r="S5" s="31"/>
-      <c r="T5" s="29">
+      <c r="R5" s="45"/>
+      <c r="S5" s="46"/>
+      <c r="T5" s="44">
         <v>14</v>
       </c>
-      <c r="U5" s="30"/>
-      <c r="V5" s="31"/>
-      <c r="W5" s="59">
+      <c r="U5" s="45"/>
+      <c r="V5" s="46"/>
+      <c r="W5" s="56">
         <v>15</v>
       </c>
-      <c r="X5" s="60"/>
-      <c r="Y5" s="61"/>
-      <c r="Z5" s="29">
+      <c r="X5" s="57"/>
+      <c r="Y5" s="58"/>
+      <c r="Z5" s="44">
         <v>16</v>
       </c>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="31"/>
-      <c r="AC5" s="29">
+      <c r="AA5" s="45"/>
+      <c r="AB5" s="46"/>
+      <c r="AC5" s="44">
         <v>17</v>
       </c>
-      <c r="AD5" s="30"/>
-      <c r="AE5" s="31"/>
-      <c r="AF5" s="29">
+      <c r="AD5" s="45"/>
+      <c r="AE5" s="46"/>
+      <c r="AF5" s="44">
         <v>18</v>
       </c>
-      <c r="AG5" s="30"/>
-      <c r="AH5" s="31"/>
-      <c r="AI5" s="29">
+      <c r="AG5" s="45"/>
+      <c r="AH5" s="46"/>
+      <c r="AI5" s="44">
         <v>19</v>
       </c>
-      <c r="AJ5" s="30"/>
-      <c r="AK5" s="31"/>
-      <c r="AL5" s="29">
+      <c r="AJ5" s="45"/>
+      <c r="AK5" s="46"/>
+      <c r="AL5" s="44">
         <v>20</v>
       </c>
-      <c r="AM5" s="30"/>
-      <c r="AN5" s="31"/>
-      <c r="AO5" s="29">
+      <c r="AM5" s="45"/>
+      <c r="AN5" s="46"/>
+      <c r="AO5" s="44">
         <v>21</v>
       </c>
-      <c r="AP5" s="30"/>
-      <c r="AQ5" s="31"/>
-      <c r="AR5" s="29">
+      <c r="AP5" s="45"/>
+      <c r="AQ5" s="46"/>
+      <c r="AR5" s="44">
         <v>22</v>
       </c>
-      <c r="AS5" s="30"/>
-      <c r="AT5" s="31"/>
-      <c r="AU5" s="29">
+      <c r="AS5" s="45"/>
+      <c r="AT5" s="46"/>
+      <c r="AU5" s="44">
         <v>23</v>
       </c>
-      <c r="AV5" s="30"/>
-      <c r="AW5" s="31"/>
-      <c r="AX5" s="50">
+      <c r="AV5" s="45"/>
+      <c r="AW5" s="46"/>
+      <c r="AX5" s="53">
         <v>24</v>
       </c>
-      <c r="AY5" s="51"/>
-      <c r="AZ5" s="52"/>
+      <c r="AY5" s="54"/>
+      <c r="AZ5" s="55"/>
     </row>
     <row r="6" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="47">
         <v>16.02</v>
       </c>
-      <c r="C6" s="34"/>
+      <c r="C6" s="49"/>
       <c r="D6" s="2">
         <v>19.02</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="47">
         <v>23.02</v>
       </c>
-      <c r="F6" s="34"/>
+      <c r="F6" s="49"/>
       <c r="G6" s="2">
         <v>26.02</v>
       </c>
-      <c r="H6" s="32">
+      <c r="H6" s="47">
         <v>2.0299999999999998</v>
       </c>
-      <c r="I6" s="34"/>
+      <c r="I6" s="49"/>
       <c r="J6" s="2">
         <v>5.03</v>
       </c>
-      <c r="K6" s="32">
+      <c r="K6" s="47">
         <v>9.0299999999999994</v>
       </c>
-      <c r="L6" s="34"/>
+      <c r="L6" s="49"/>
       <c r="M6" s="2">
         <v>12.03</v>
       </c>
-      <c r="N6" s="32">
+      <c r="N6" s="47">
         <v>16.03</v>
       </c>
-      <c r="O6" s="34"/>
+      <c r="O6" s="49"/>
       <c r="P6" s="2">
         <v>19.03</v>
       </c>
-      <c r="Q6" s="32">
+      <c r="Q6" s="47">
         <v>23.03</v>
       </c>
-      <c r="R6" s="34"/>
+      <c r="R6" s="49"/>
       <c r="S6" s="2">
         <v>26.03</v>
       </c>
-      <c r="T6" s="32">
+      <c r="T6" s="47">
         <v>30.03</v>
       </c>
-      <c r="U6" s="34"/>
+      <c r="U6" s="49"/>
       <c r="V6" s="2">
         <v>2.04</v>
       </c>
-      <c r="W6" s="62">
+      <c r="W6" s="59">
         <v>6.04</v>
       </c>
-      <c r="X6" s="63"/>
+      <c r="X6" s="60"/>
       <c r="Y6" s="3">
         <v>9.0399999999999991</v>
       </c>
-      <c r="Z6" s="32">
+      <c r="Z6" s="47">
         <v>13.04</v>
       </c>
-      <c r="AA6" s="34"/>
+      <c r="AA6" s="49"/>
       <c r="AB6" s="2">
         <v>16.04</v>
       </c>
-      <c r="AC6" s="32">
+      <c r="AC6" s="47">
         <v>20.04</v>
       </c>
-      <c r="AD6" s="34"/>
+      <c r="AD6" s="49"/>
       <c r="AE6" s="2">
         <v>23.04</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="47">
         <v>27.04</v>
       </c>
-      <c r="AG6" s="34"/>
+      <c r="AG6" s="49"/>
       <c r="AH6" s="2">
         <v>30.04</v>
       </c>
-      <c r="AI6" s="32">
+      <c r="AI6" s="47">
         <v>4.05</v>
       </c>
-      <c r="AJ6" s="34"/>
+      <c r="AJ6" s="49"/>
       <c r="AK6" s="2">
         <v>7.05</v>
       </c>
-      <c r="AL6" s="32">
+      <c r="AL6" s="47">
         <v>11.05</v>
       </c>
-      <c r="AM6" s="34"/>
+      <c r="AM6" s="49"/>
       <c r="AN6" s="2">
         <v>14.05</v>
       </c>
-      <c r="AO6" s="32">
+      <c r="AO6" s="47">
         <v>18.05</v>
       </c>
-      <c r="AP6" s="34"/>
+      <c r="AP6" s="49"/>
       <c r="AQ6" s="2">
         <v>21.05</v>
       </c>
-      <c r="AR6" s="32">
+      <c r="AR6" s="47">
         <v>25.05</v>
       </c>
-      <c r="AS6" s="34"/>
+      <c r="AS6" s="49"/>
       <c r="AT6" s="2">
         <v>28.05</v>
       </c>
-      <c r="AU6" s="32">
+      <c r="AU6" s="47">
         <v>1.06</v>
       </c>
-      <c r="AV6" s="34"/>
+      <c r="AV6" s="49"/>
       <c r="AW6" s="2">
         <v>4.0599999999999996</v>
       </c>
-      <c r="AX6" s="32">
+      <c r="AX6" s="47">
         <v>8.06</v>
       </c>
-      <c r="AY6" s="34"/>
+      <c r="AY6" s="49"/>
       <c r="AZ6" s="2">
         <v>11.06</v>
       </c>
@@ -6055,32 +6054,32 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="39" t="s">
+      <c r="H8" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="40"/>
-      <c r="J8" s="41"/>
-      <c r="K8" s="64" t="s">
+      <c r="I8" s="42"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="61" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="65"/>
-      <c r="M8" s="66"/>
-      <c r="N8" s="53" t="s">
+      <c r="L8" s="62"/>
+      <c r="M8" s="63"/>
+      <c r="N8" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="O8" s="54"/>
-      <c r="P8" s="55"/>
+      <c r="O8" s="65"/>
+      <c r="P8" s="66"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
-      <c r="W8" s="56" t="s">
+      <c r="W8" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="X8" s="57"/>
-      <c r="Y8" s="58"/>
+      <c r="X8" s="51"/>
+      <c r="Y8" s="52"/>
       <c r="Z8" s="4"/>
       <c r="AA8" s="4"/>
       <c r="AB8" s="4"/>
@@ -6105,11 +6104,11 @@
       <c r="AU8" s="4"/>
       <c r="AV8" s="4"/>
       <c r="AW8" s="4"/>
-      <c r="AX8" s="39" t="s">
+      <c r="AX8" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="AY8" s="40"/>
-      <c r="AZ8" s="41"/>
+      <c r="AY8" s="42"/>
+      <c r="AZ8" s="43"/>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -7980,7 +7979,7 @@
       <c r="AZ42" s="7"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A43" s="44" t="s">
+      <c r="A43" s="39" t="s">
         <v>40</v>
       </c>
       <c r="B43" s="5"/>
@@ -8036,7 +8035,7 @@
       <c r="AZ43" s="5"/>
     </row>
     <row r="44" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="45"/>
+      <c r="A44" s="40"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -8201,6 +8200,54 @@
     </row>
   </sheetData>
   <mergeCells count="64">
+    <mergeCell ref="AU5:AW5"/>
+    <mergeCell ref="AU6:AV6"/>
+    <mergeCell ref="AX5:AZ5"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="AO6:AP6"/>
+    <mergeCell ref="AR5:AT5"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="AC6:AD6"/>
+    <mergeCell ref="AF5:AH5"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H6:I6"/>
     <mergeCell ref="AX8:AZ8"/>
     <mergeCell ref="W8:Y8"/>
     <mergeCell ref="K5:M5"/>
@@ -8217,54 +8264,6 @@
     <mergeCell ref="Z6:AA6"/>
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="AC5:AE5"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="AC6:AD6"/>
-    <mergeCell ref="AF5:AH5"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="AU5:AW5"/>
-    <mergeCell ref="AU6:AV6"/>
-    <mergeCell ref="AX5:AZ5"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="AO5:AQ5"/>
-    <mergeCell ref="AO6:AP6"/>
-    <mergeCell ref="AR5:AT5"/>
-    <mergeCell ref="AR6:AS6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Electronic design redaction, Annexes
</commit_message>
<xml_diff>
--- a/A_Documentation/Planning.xlsx
+++ b/A_Documentation/Planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\Documents\Repositories\Self-Balancing-Bot\A_Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13006F8B-8917-450D-B57A-9B2B7D63ACDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5E800AC-3DC9-4BA5-9D37-8A449115D7D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -667,51 +667,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -730,14 +685,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -747,6 +738,24 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -770,15 +779,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1208,12 +1208,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="30"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="47"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -1221,29 +1221,29 @@
       <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="31" t="s">
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="32"/>
+      <c r="G2" s="49"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31" t="s">
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="32"/>
+      <c r="G3" s="49"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:61" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -1251,165 +1251,165 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="33" t="s">
+      <c r="F4" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="34"/>
+      <c r="G4" s="43"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="44">
+      <c r="B5" s="29">
         <v>25</v>
       </c>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="45"/>
-      <c r="I5" s="45"/>
-      <c r="J5" s="45"/>
-      <c r="K5" s="46"/>
-      <c r="L5" s="44">
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="29">
         <v>26</v>
       </c>
-      <c r="M5" s="45"/>
-      <c r="N5" s="45"/>
-      <c r="O5" s="45"/>
-      <c r="P5" s="45"/>
-      <c r="Q5" s="45"/>
-      <c r="R5" s="45"/>
-      <c r="S5" s="45"/>
-      <c r="T5" s="45"/>
-      <c r="U5" s="46"/>
-      <c r="V5" s="44">
+      <c r="M5" s="30"/>
+      <c r="N5" s="30"/>
+      <c r="O5" s="30"/>
+      <c r="P5" s="30"/>
+      <c r="Q5" s="30"/>
+      <c r="R5" s="30"/>
+      <c r="S5" s="30"/>
+      <c r="T5" s="30"/>
+      <c r="U5" s="31"/>
+      <c r="V5" s="29">
         <v>27</v>
       </c>
-      <c r="W5" s="45"/>
-      <c r="X5" s="45"/>
-      <c r="Y5" s="45"/>
-      <c r="Z5" s="45"/>
-      <c r="AA5" s="45"/>
-      <c r="AB5" s="45"/>
-      <c r="AC5" s="45"/>
-      <c r="AD5" s="45"/>
-      <c r="AE5" s="46"/>
-      <c r="AF5" s="44">
+      <c r="W5" s="30"/>
+      <c r="X5" s="30"/>
+      <c r="Y5" s="30"/>
+      <c r="Z5" s="30"/>
+      <c r="AA5" s="30"/>
+      <c r="AB5" s="30"/>
+      <c r="AC5" s="30"/>
+      <c r="AD5" s="30"/>
+      <c r="AE5" s="31"/>
+      <c r="AF5" s="29">
         <v>28</v>
       </c>
-      <c r="AG5" s="45"/>
-      <c r="AH5" s="45"/>
-      <c r="AI5" s="45"/>
-      <c r="AJ5" s="45"/>
-      <c r="AK5" s="45"/>
-      <c r="AL5" s="45"/>
-      <c r="AM5" s="45"/>
-      <c r="AN5" s="45"/>
-      <c r="AO5" s="46"/>
-      <c r="AP5" s="44">
+      <c r="AG5" s="30"/>
+      <c r="AH5" s="30"/>
+      <c r="AI5" s="30"/>
+      <c r="AJ5" s="30"/>
+      <c r="AK5" s="30"/>
+      <c r="AL5" s="30"/>
+      <c r="AM5" s="30"/>
+      <c r="AN5" s="30"/>
+      <c r="AO5" s="31"/>
+      <c r="AP5" s="29">
         <v>29</v>
       </c>
-      <c r="AQ5" s="45"/>
-      <c r="AR5" s="45"/>
-      <c r="AS5" s="45"/>
-      <c r="AT5" s="45"/>
-      <c r="AU5" s="45"/>
-      <c r="AV5" s="45"/>
-      <c r="AW5" s="45"/>
-      <c r="AX5" s="45"/>
-      <c r="AY5" s="46"/>
-      <c r="AZ5" s="44">
+      <c r="AQ5" s="30"/>
+      <c r="AR5" s="30"/>
+      <c r="AS5" s="30"/>
+      <c r="AT5" s="30"/>
+      <c r="AU5" s="30"/>
+      <c r="AV5" s="30"/>
+      <c r="AW5" s="30"/>
+      <c r="AX5" s="30"/>
+      <c r="AY5" s="31"/>
+      <c r="AZ5" s="29">
         <v>30</v>
       </c>
-      <c r="BA5" s="45"/>
-      <c r="BB5" s="45"/>
-      <c r="BC5" s="45"/>
-      <c r="BD5" s="45"/>
-      <c r="BE5" s="45"/>
-      <c r="BF5" s="45"/>
-      <c r="BG5" s="45"/>
-      <c r="BH5" s="45"/>
-      <c r="BI5" s="46"/>
+      <c r="BA5" s="30"/>
+      <c r="BB5" s="30"/>
+      <c r="BC5" s="30"/>
+      <c r="BD5" s="30"/>
+      <c r="BE5" s="30"/>
+      <c r="BF5" s="30"/>
+      <c r="BG5" s="30"/>
+      <c r="BH5" s="30"/>
+      <c r="BI5" s="31"/>
     </row>
     <row r="6" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="49"/>
-      <c r="L6" s="47" t="s">
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="34"/>
+      <c r="L6" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="48"/>
-      <c r="N6" s="48"/>
-      <c r="O6" s="48"/>
-      <c r="P6" s="48"/>
-      <c r="Q6" s="48"/>
-      <c r="R6" s="48"/>
-      <c r="S6" s="48"/>
-      <c r="T6" s="48"/>
-      <c r="U6" s="49"/>
-      <c r="V6" s="47" t="s">
+      <c r="M6" s="33"/>
+      <c r="N6" s="33"/>
+      <c r="O6" s="33"/>
+      <c r="P6" s="33"/>
+      <c r="Q6" s="33"/>
+      <c r="R6" s="33"/>
+      <c r="S6" s="33"/>
+      <c r="T6" s="33"/>
+      <c r="U6" s="34"/>
+      <c r="V6" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="W6" s="48"/>
-      <c r="X6" s="48"/>
-      <c r="Y6" s="48"/>
-      <c r="Z6" s="48"/>
-      <c r="AA6" s="48"/>
-      <c r="AB6" s="48"/>
-      <c r="AC6" s="48"/>
-      <c r="AD6" s="48"/>
-      <c r="AE6" s="49"/>
-      <c r="AF6" s="47" t="s">
+      <c r="W6" s="33"/>
+      <c r="X6" s="33"/>
+      <c r="Y6" s="33"/>
+      <c r="Z6" s="33"/>
+      <c r="AA6" s="33"/>
+      <c r="AB6" s="33"/>
+      <c r="AC6" s="33"/>
+      <c r="AD6" s="33"/>
+      <c r="AE6" s="34"/>
+      <c r="AF6" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="AG6" s="48"/>
-      <c r="AH6" s="48"/>
-      <c r="AI6" s="48"/>
-      <c r="AJ6" s="48"/>
-      <c r="AK6" s="48"/>
-      <c r="AL6" s="48"/>
-      <c r="AM6" s="48"/>
-      <c r="AN6" s="48"/>
-      <c r="AO6" s="49"/>
-      <c r="AP6" s="47" t="s">
+      <c r="AG6" s="33"/>
+      <c r="AH6" s="33"/>
+      <c r="AI6" s="33"/>
+      <c r="AJ6" s="33"/>
+      <c r="AK6" s="33"/>
+      <c r="AL6" s="33"/>
+      <c r="AM6" s="33"/>
+      <c r="AN6" s="33"/>
+      <c r="AO6" s="34"/>
+      <c r="AP6" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="AQ6" s="48"/>
-      <c r="AR6" s="48"/>
-      <c r="AS6" s="48"/>
-      <c r="AT6" s="48"/>
-      <c r="AU6" s="48"/>
-      <c r="AV6" s="48"/>
-      <c r="AW6" s="48"/>
-      <c r="AX6" s="48"/>
-      <c r="AY6" s="49"/>
-      <c r="AZ6" s="47" t="s">
+      <c r="AQ6" s="33"/>
+      <c r="AR6" s="33"/>
+      <c r="AS6" s="33"/>
+      <c r="AT6" s="33"/>
+      <c r="AU6" s="33"/>
+      <c r="AV6" s="33"/>
+      <c r="AW6" s="33"/>
+      <c r="AX6" s="33"/>
+      <c r="AY6" s="34"/>
+      <c r="AZ6" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="BA6" s="48"/>
-      <c r="BB6" s="48"/>
-      <c r="BC6" s="48"/>
-      <c r="BD6" s="48"/>
-      <c r="BE6" s="48"/>
-      <c r="BF6" s="48"/>
-      <c r="BG6" s="48"/>
-      <c r="BH6" s="48"/>
-      <c r="BI6" s="49"/>
+      <c r="BA6" s="33"/>
+      <c r="BB6" s="33"/>
+      <c r="BC6" s="33"/>
+      <c r="BD6" s="33"/>
+      <c r="BE6" s="33"/>
+      <c r="BF6" s="33"/>
+      <c r="BG6" s="33"/>
+      <c r="BH6" s="33"/>
+      <c r="BI6" s="34"/>
     </row>
     <row r="7" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -1600,18 +1600,18 @@
       <c r="A8" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="AZ8" s="41" t="s">
+      <c r="AZ8" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="BA8" s="42"/>
-      <c r="BB8" s="42"/>
-      <c r="BC8" s="42"/>
-      <c r="BD8" s="42"/>
-      <c r="BE8" s="42"/>
-      <c r="BF8" s="42"/>
-      <c r="BG8" s="42"/>
-      <c r="BH8" s="42"/>
-      <c r="BI8" s="43"/>
+      <c r="BA8" s="40"/>
+      <c r="BB8" s="40"/>
+      <c r="BC8" s="40"/>
+      <c r="BD8" s="40"/>
+      <c r="BE8" s="40"/>
+      <c r="BF8" s="40"/>
+      <c r="BG8" s="40"/>
+      <c r="BH8" s="40"/>
+      <c r="BI8" s="41"/>
     </row>
     <row r="9" spans="1:61" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -2345,11 +2345,11 @@
       <c r="X20" s="10"/>
       <c r="Y20" s="10"/>
       <c r="Z20" s="10"/>
-      <c r="AA20" s="7"/>
-      <c r="AB20" s="7"/>
-      <c r="AC20" s="7"/>
-      <c r="AD20" s="7"/>
-      <c r="AE20" s="7"/>
+      <c r="AA20" s="10"/>
+      <c r="AB20" s="10"/>
+      <c r="AC20" s="10"/>
+      <c r="AD20" s="10"/>
+      <c r="AE20" s="10"/>
       <c r="AF20" s="7"/>
       <c r="AG20" s="7"/>
       <c r="AH20" s="7"/>
@@ -2475,9 +2475,9 @@
       <c r="Z22" s="7"/>
       <c r="AA22" s="7"/>
       <c r="AB22" s="7"/>
-      <c r="AC22" s="7"/>
-      <c r="AD22" s="7"/>
-      <c r="AE22" s="7"/>
+      <c r="AC22" s="10"/>
+      <c r="AD22" s="10"/>
+      <c r="AE22" s="10"/>
       <c r="AF22" s="7"/>
       <c r="AG22" s="7"/>
       <c r="AH22" s="7"/>
@@ -3276,7 +3276,7 @@
       <c r="BI34" s="7"/>
     </row>
     <row r="35" spans="1:61" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="39" t="s">
+      <c r="A35" s="44" t="s">
         <v>40</v>
       </c>
       <c r="B35" s="5"/>
@@ -3341,7 +3341,7 @@
       <c r="BI35" s="24"/>
     </row>
     <row r="36" spans="1:61" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="40"/>
+      <c r="A36" s="45"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
@@ -5549,35 +5549,11 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="B5:K5"/>
-    <mergeCell ref="AZ6:BI6"/>
-    <mergeCell ref="L5:U5"/>
-    <mergeCell ref="V5:AE5"/>
-    <mergeCell ref="AF5:AO5"/>
-    <mergeCell ref="AP5:AY5"/>
-    <mergeCell ref="AZ5:BI5"/>
-    <mergeCell ref="B6:K6"/>
-    <mergeCell ref="L6:U6"/>
-    <mergeCell ref="V6:AE6"/>
-    <mergeCell ref="AF6:AO6"/>
-    <mergeCell ref="AP6:AY6"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="AZ8:BI8"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A61:A62"/>
     <mergeCell ref="A63:A64"/>
@@ -5594,11 +5570,35 @@
     <mergeCell ref="A33:A34"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="AZ8:BI8"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="AZ6:BI6"/>
+    <mergeCell ref="L5:U5"/>
+    <mergeCell ref="V5:AE5"/>
+    <mergeCell ref="AF5:AO5"/>
+    <mergeCell ref="AP5:AY5"/>
+    <mergeCell ref="AZ5:BI5"/>
+    <mergeCell ref="B6:K6"/>
+    <mergeCell ref="L6:U6"/>
+    <mergeCell ref="V6:AE6"/>
+    <mergeCell ref="AF6:AO6"/>
+    <mergeCell ref="AP6:AY6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5618,12 +5618,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="30"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="47"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -5642,29 +5642,29 @@
       <c r="Q1" s="17"/>
     </row>
     <row r="2" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="31" t="s">
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="32"/>
+      <c r="G2" s="49"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31" t="s">
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="32"/>
+      <c r="G3" s="49"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:52" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -5672,222 +5672,222 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="33" t="s">
+      <c r="F4" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="34"/>
+      <c r="G4" s="43"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="44">
+      <c r="B5" s="29">
         <v>8</v>
       </c>
-      <c r="C5" s="45"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="44">
+      <c r="C5" s="30"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="29">
         <v>9</v>
       </c>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
-      <c r="H5" s="53" t="s">
+      <c r="F5" s="30"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="54"/>
-      <c r="J5" s="55"/>
-      <c r="K5" s="44">
+      <c r="I5" s="51"/>
+      <c r="J5" s="52"/>
+      <c r="K5" s="29">
         <v>11</v>
       </c>
-      <c r="L5" s="45"/>
-      <c r="M5" s="46"/>
-      <c r="N5" s="53" t="s">
+      <c r="L5" s="30"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="54"/>
-      <c r="P5" s="55"/>
-      <c r="Q5" s="44">
+      <c r="O5" s="51"/>
+      <c r="P5" s="52"/>
+      <c r="Q5" s="29">
         <v>13</v>
       </c>
-      <c r="R5" s="45"/>
-      <c r="S5" s="46"/>
-      <c r="T5" s="44">
+      <c r="R5" s="30"/>
+      <c r="S5" s="31"/>
+      <c r="T5" s="29">
         <v>14</v>
       </c>
-      <c r="U5" s="45"/>
-      <c r="V5" s="46"/>
-      <c r="W5" s="56">
+      <c r="U5" s="30"/>
+      <c r="V5" s="31"/>
+      <c r="W5" s="59">
         <v>15</v>
       </c>
-      <c r="X5" s="57"/>
-      <c r="Y5" s="58"/>
-      <c r="Z5" s="44">
+      <c r="X5" s="60"/>
+      <c r="Y5" s="61"/>
+      <c r="Z5" s="29">
         <v>16</v>
       </c>
-      <c r="AA5" s="45"/>
-      <c r="AB5" s="46"/>
-      <c r="AC5" s="44">
+      <c r="AA5" s="30"/>
+      <c r="AB5" s="31"/>
+      <c r="AC5" s="29">
         <v>17</v>
       </c>
-      <c r="AD5" s="45"/>
-      <c r="AE5" s="46"/>
-      <c r="AF5" s="44">
+      <c r="AD5" s="30"/>
+      <c r="AE5" s="31"/>
+      <c r="AF5" s="29">
         <v>18</v>
       </c>
-      <c r="AG5" s="45"/>
-      <c r="AH5" s="46"/>
-      <c r="AI5" s="44">
+      <c r="AG5" s="30"/>
+      <c r="AH5" s="31"/>
+      <c r="AI5" s="29">
         <v>19</v>
       </c>
-      <c r="AJ5" s="45"/>
-      <c r="AK5" s="46"/>
-      <c r="AL5" s="44">
+      <c r="AJ5" s="30"/>
+      <c r="AK5" s="31"/>
+      <c r="AL5" s="29">
         <v>20</v>
       </c>
-      <c r="AM5" s="45"/>
-      <c r="AN5" s="46"/>
-      <c r="AO5" s="44">
+      <c r="AM5" s="30"/>
+      <c r="AN5" s="31"/>
+      <c r="AO5" s="29">
         <v>21</v>
       </c>
-      <c r="AP5" s="45"/>
-      <c r="AQ5" s="46"/>
-      <c r="AR5" s="44">
+      <c r="AP5" s="30"/>
+      <c r="AQ5" s="31"/>
+      <c r="AR5" s="29">
         <v>22</v>
       </c>
-      <c r="AS5" s="45"/>
-      <c r="AT5" s="46"/>
-      <c r="AU5" s="44">
+      <c r="AS5" s="30"/>
+      <c r="AT5" s="31"/>
+      <c r="AU5" s="29">
         <v>23</v>
       </c>
-      <c r="AV5" s="45"/>
-      <c r="AW5" s="46"/>
-      <c r="AX5" s="53">
+      <c r="AV5" s="30"/>
+      <c r="AW5" s="31"/>
+      <c r="AX5" s="50">
         <v>24</v>
       </c>
-      <c r="AY5" s="54"/>
-      <c r="AZ5" s="55"/>
+      <c r="AY5" s="51"/>
+      <c r="AZ5" s="52"/>
     </row>
     <row r="6" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="47">
+      <c r="B6" s="32">
         <v>16.02</v>
       </c>
-      <c r="C6" s="49"/>
+      <c r="C6" s="34"/>
       <c r="D6" s="2">
         <v>19.02</v>
       </c>
-      <c r="E6" s="47">
+      <c r="E6" s="32">
         <v>23.02</v>
       </c>
-      <c r="F6" s="49"/>
+      <c r="F6" s="34"/>
       <c r="G6" s="2">
         <v>26.02</v>
       </c>
-      <c r="H6" s="47">
+      <c r="H6" s="32">
         <v>2.0299999999999998</v>
       </c>
-      <c r="I6" s="49"/>
+      <c r="I6" s="34"/>
       <c r="J6" s="2">
         <v>5.03</v>
       </c>
-      <c r="K6" s="47">
+      <c r="K6" s="32">
         <v>9.0299999999999994</v>
       </c>
-      <c r="L6" s="49"/>
+      <c r="L6" s="34"/>
       <c r="M6" s="2">
         <v>12.03</v>
       </c>
-      <c r="N6" s="47">
+      <c r="N6" s="32">
         <v>16.03</v>
       </c>
-      <c r="O6" s="49"/>
+      <c r="O6" s="34"/>
       <c r="P6" s="2">
         <v>19.03</v>
       </c>
-      <c r="Q6" s="47">
+      <c r="Q6" s="32">
         <v>23.03</v>
       </c>
-      <c r="R6" s="49"/>
+      <c r="R6" s="34"/>
       <c r="S6" s="2">
         <v>26.03</v>
       </c>
-      <c r="T6" s="47">
+      <c r="T6" s="32">
         <v>30.03</v>
       </c>
-      <c r="U6" s="49"/>
+      <c r="U6" s="34"/>
       <c r="V6" s="2">
         <v>2.04</v>
       </c>
-      <c r="W6" s="59">
+      <c r="W6" s="62">
         <v>6.04</v>
       </c>
-      <c r="X6" s="60"/>
+      <c r="X6" s="63"/>
       <c r="Y6" s="3">
         <v>9.0399999999999991</v>
       </c>
-      <c r="Z6" s="47">
+      <c r="Z6" s="32">
         <v>13.04</v>
       </c>
-      <c r="AA6" s="49"/>
+      <c r="AA6" s="34"/>
       <c r="AB6" s="2">
         <v>16.04</v>
       </c>
-      <c r="AC6" s="47">
+      <c r="AC6" s="32">
         <v>20.04</v>
       </c>
-      <c r="AD6" s="49"/>
+      <c r="AD6" s="34"/>
       <c r="AE6" s="2">
         <v>23.04</v>
       </c>
-      <c r="AF6" s="47">
+      <c r="AF6" s="32">
         <v>27.04</v>
       </c>
-      <c r="AG6" s="49"/>
+      <c r="AG6" s="34"/>
       <c r="AH6" s="2">
         <v>30.04</v>
       </c>
-      <c r="AI6" s="47">
+      <c r="AI6" s="32">
         <v>4.05</v>
       </c>
-      <c r="AJ6" s="49"/>
+      <c r="AJ6" s="34"/>
       <c r="AK6" s="2">
         <v>7.05</v>
       </c>
-      <c r="AL6" s="47">
+      <c r="AL6" s="32">
         <v>11.05</v>
       </c>
-      <c r="AM6" s="49"/>
+      <c r="AM6" s="34"/>
       <c r="AN6" s="2">
         <v>14.05</v>
       </c>
-      <c r="AO6" s="47">
+      <c r="AO6" s="32">
         <v>18.05</v>
       </c>
-      <c r="AP6" s="49"/>
+      <c r="AP6" s="34"/>
       <c r="AQ6" s="2">
         <v>21.05</v>
       </c>
-      <c r="AR6" s="47">
+      <c r="AR6" s="32">
         <v>25.05</v>
       </c>
-      <c r="AS6" s="49"/>
+      <c r="AS6" s="34"/>
       <c r="AT6" s="2">
         <v>28.05</v>
       </c>
-      <c r="AU6" s="47">
+      <c r="AU6" s="32">
         <v>1.06</v>
       </c>
-      <c r="AV6" s="49"/>
+      <c r="AV6" s="34"/>
       <c r="AW6" s="2">
         <v>4.0599999999999996</v>
       </c>
-      <c r="AX6" s="47">
+      <c r="AX6" s="32">
         <v>8.06</v>
       </c>
-      <c r="AY6" s="49"/>
+      <c r="AY6" s="34"/>
       <c r="AZ6" s="2">
         <v>11.06</v>
       </c>
@@ -6054,32 +6054,32 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="41" t="s">
+      <c r="H8" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="42"/>
-      <c r="J8" s="43"/>
-      <c r="K8" s="61" t="s">
+      <c r="I8" s="40"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="64" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="62"/>
-      <c r="M8" s="63"/>
-      <c r="N8" s="64" t="s">
+      <c r="L8" s="65"/>
+      <c r="M8" s="66"/>
+      <c r="N8" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="O8" s="65"/>
-      <c r="P8" s="66"/>
+      <c r="O8" s="54"/>
+      <c r="P8" s="55"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
-      <c r="W8" s="50" t="s">
+      <c r="W8" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="X8" s="51"/>
-      <c r="Y8" s="52"/>
+      <c r="X8" s="57"/>
+      <c r="Y8" s="58"/>
       <c r="Z8" s="4"/>
       <c r="AA8" s="4"/>
       <c r="AB8" s="4"/>
@@ -6104,11 +6104,11 @@
       <c r="AU8" s="4"/>
       <c r="AV8" s="4"/>
       <c r="AW8" s="4"/>
-      <c r="AX8" s="41" t="s">
+      <c r="AX8" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="AY8" s="42"/>
-      <c r="AZ8" s="43"/>
+      <c r="AY8" s="40"/>
+      <c r="AZ8" s="41"/>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -7979,7 +7979,7 @@
       <c r="AZ42" s="7"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A43" s="39" t="s">
+      <c r="A43" s="44" t="s">
         <v>40</v>
       </c>
       <c r="B43" s="5"/>
@@ -8035,7 +8035,7 @@
       <c r="AZ43" s="5"/>
     </row>
     <row r="44" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="40"/>
+      <c r="A44" s="45"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -8200,54 +8200,6 @@
     </row>
   </sheetData>
   <mergeCells count="64">
-    <mergeCell ref="AU5:AW5"/>
-    <mergeCell ref="AU6:AV6"/>
-    <mergeCell ref="AX5:AZ5"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="AO5:AQ5"/>
-    <mergeCell ref="AO6:AP6"/>
-    <mergeCell ref="AR5:AT5"/>
-    <mergeCell ref="AR6:AS6"/>
-    <mergeCell ref="AC6:AD6"/>
-    <mergeCell ref="AF5:AH5"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H6:I6"/>
     <mergeCell ref="AX8:AZ8"/>
     <mergeCell ref="W8:Y8"/>
     <mergeCell ref="K5:M5"/>
@@ -8264,6 +8216,54 @@
     <mergeCell ref="Z6:AA6"/>
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="AC5:AE5"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="AC6:AD6"/>
+    <mergeCell ref="AF5:AH5"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="AU5:AW5"/>
+    <mergeCell ref="AU6:AV6"/>
+    <mergeCell ref="AX5:AZ5"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="AO6:AP6"/>
+    <mergeCell ref="AR5:AT5"/>
+    <mergeCell ref="AR6:AS6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
End of electronic design's rapport
</commit_message>
<xml_diff>
--- a/A_Documentation/Planning.xlsx
+++ b/A_Documentation/Planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\Documents\Repositories\Self-Balancing-Bot\A_Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5E800AC-3DC9-4BA5-9D37-8A449115D7D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B54DB4C-92FB-4020-A189-6050DC35A09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="57">
   <si>
     <t>Semaines</t>
   </si>
@@ -221,9 +221,6 @@
   </si>
   <si>
     <t>Rédaction rapport: Conclusion, Mesures</t>
-  </si>
-  <si>
-    <t>Résèrve</t>
   </si>
   <si>
     <t>Test Autonomie</t>
@@ -1743,7 +1740,7 @@
     </row>
     <row r="11" spans="1:61" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -2127,7 +2124,7 @@
     </row>
     <row r="17" spans="1:61" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A17" s="37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -2255,7 +2252,7 @@
     </row>
     <row r="19" spans="1:61" s="26" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19" s="37" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -2353,7 +2350,7 @@
       <c r="AF20" s="7"/>
       <c r="AG20" s="7"/>
       <c r="AH20" s="7"/>
-      <c r="AI20" s="7"/>
+      <c r="AI20" s="10"/>
       <c r="AJ20" s="7"/>
       <c r="AK20" s="7"/>
       <c r="AL20" s="7"/>
@@ -2478,9 +2475,9 @@
       <c r="AC22" s="10"/>
       <c r="AD22" s="10"/>
       <c r="AE22" s="10"/>
-      <c r="AF22" s="7"/>
-      <c r="AG22" s="7"/>
-      <c r="AH22" s="7"/>
+      <c r="AF22" s="10"/>
+      <c r="AG22" s="10"/>
+      <c r="AH22" s="10"/>
       <c r="AI22" s="7"/>
       <c r="AJ22" s="7"/>
       <c r="AK22" s="7"/>
@@ -2639,7 +2636,7 @@
     </row>
     <row r="25" spans="1:61" s="28" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A25" s="37" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -2767,7 +2764,7 @@
     </row>
     <row r="27" spans="1:61" s="28" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A27" s="37" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -2895,7 +2892,7 @@
     </row>
     <row r="29" spans="1:61" s="28" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A29" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -3023,7 +3020,7 @@
     </row>
     <row r="31" spans="1:61" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31" s="37" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>

</xml_diff>

<commit_message>
Redaction of Embedded system programmation, Modified HTML title, refactor TMC2226.cpp
</commit_message>
<xml_diff>
--- a/A_Documentation/Planning.xlsx
+++ b/A_Documentation/Planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\Documents\Repositories\Self-Balancing-Bot\A_Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B54DB4C-92FB-4020-A189-6050DC35A09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E713F251-6174-40CF-86AB-4ABD5C2131B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -664,6 +664,51 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -682,50 +727,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -735,24 +744,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -776,6 +767,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1205,12 +1205,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="47"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -1218,29 +1218,29 @@
       <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="48" t="s">
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="49"/>
+      <c r="G2" s="32"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="48" t="s">
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="49"/>
+      <c r="G3" s="32"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:61" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -1248,165 +1248,165 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="42" t="s">
+      <c r="F4" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="43"/>
+      <c r="G4" s="34"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="44">
         <v>25</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="31"/>
-      <c r="L5" s="29">
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="46"/>
+      <c r="L5" s="44">
         <v>26</v>
       </c>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
-      <c r="P5" s="30"/>
-      <c r="Q5" s="30"/>
-      <c r="R5" s="30"/>
-      <c r="S5" s="30"/>
-      <c r="T5" s="30"/>
-      <c r="U5" s="31"/>
-      <c r="V5" s="29">
+      <c r="M5" s="45"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="45"/>
+      <c r="P5" s="45"/>
+      <c r="Q5" s="45"/>
+      <c r="R5" s="45"/>
+      <c r="S5" s="45"/>
+      <c r="T5" s="45"/>
+      <c r="U5" s="46"/>
+      <c r="V5" s="44">
         <v>27</v>
       </c>
-      <c r="W5" s="30"/>
-      <c r="X5" s="30"/>
-      <c r="Y5" s="30"/>
-      <c r="Z5" s="30"/>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="30"/>
-      <c r="AC5" s="30"/>
-      <c r="AD5" s="30"/>
-      <c r="AE5" s="31"/>
-      <c r="AF5" s="29">
+      <c r="W5" s="45"/>
+      <c r="X5" s="45"/>
+      <c r="Y5" s="45"/>
+      <c r="Z5" s="45"/>
+      <c r="AA5" s="45"/>
+      <c r="AB5" s="45"/>
+      <c r="AC5" s="45"/>
+      <c r="AD5" s="45"/>
+      <c r="AE5" s="46"/>
+      <c r="AF5" s="44">
         <v>28</v>
       </c>
-      <c r="AG5" s="30"/>
-      <c r="AH5" s="30"/>
-      <c r="AI5" s="30"/>
-      <c r="AJ5" s="30"/>
-      <c r="AK5" s="30"/>
-      <c r="AL5" s="30"/>
-      <c r="AM5" s="30"/>
-      <c r="AN5" s="30"/>
-      <c r="AO5" s="31"/>
-      <c r="AP5" s="29">
+      <c r="AG5" s="45"/>
+      <c r="AH5" s="45"/>
+      <c r="AI5" s="45"/>
+      <c r="AJ5" s="45"/>
+      <c r="AK5" s="45"/>
+      <c r="AL5" s="45"/>
+      <c r="AM5" s="45"/>
+      <c r="AN5" s="45"/>
+      <c r="AO5" s="46"/>
+      <c r="AP5" s="44">
         <v>29</v>
       </c>
-      <c r="AQ5" s="30"/>
-      <c r="AR5" s="30"/>
-      <c r="AS5" s="30"/>
-      <c r="AT5" s="30"/>
-      <c r="AU5" s="30"/>
-      <c r="AV5" s="30"/>
-      <c r="AW5" s="30"/>
-      <c r="AX5" s="30"/>
-      <c r="AY5" s="31"/>
-      <c r="AZ5" s="29">
+      <c r="AQ5" s="45"/>
+      <c r="AR5" s="45"/>
+      <c r="AS5" s="45"/>
+      <c r="AT5" s="45"/>
+      <c r="AU5" s="45"/>
+      <c r="AV5" s="45"/>
+      <c r="AW5" s="45"/>
+      <c r="AX5" s="45"/>
+      <c r="AY5" s="46"/>
+      <c r="AZ5" s="44">
         <v>30</v>
       </c>
-      <c r="BA5" s="30"/>
-      <c r="BB5" s="30"/>
-      <c r="BC5" s="30"/>
-      <c r="BD5" s="30"/>
-      <c r="BE5" s="30"/>
-      <c r="BF5" s="30"/>
-      <c r="BG5" s="30"/>
-      <c r="BH5" s="30"/>
-      <c r="BI5" s="31"/>
+      <c r="BA5" s="45"/>
+      <c r="BB5" s="45"/>
+      <c r="BC5" s="45"/>
+      <c r="BD5" s="45"/>
+      <c r="BE5" s="45"/>
+      <c r="BF5" s="45"/>
+      <c r="BG5" s="45"/>
+      <c r="BH5" s="45"/>
+      <c r="BI5" s="46"/>
     </row>
     <row r="6" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="33"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="32" t="s">
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="33"/>
-      <c r="N6" s="33"/>
-      <c r="O6" s="33"/>
-      <c r="P6" s="33"/>
-      <c r="Q6" s="33"/>
-      <c r="R6" s="33"/>
-      <c r="S6" s="33"/>
-      <c r="T6" s="33"/>
-      <c r="U6" s="34"/>
-      <c r="V6" s="32" t="s">
+      <c r="M6" s="48"/>
+      <c r="N6" s="48"/>
+      <c r="O6" s="48"/>
+      <c r="P6" s="48"/>
+      <c r="Q6" s="48"/>
+      <c r="R6" s="48"/>
+      <c r="S6" s="48"/>
+      <c r="T6" s="48"/>
+      <c r="U6" s="49"/>
+      <c r="V6" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="W6" s="33"/>
-      <c r="X6" s="33"/>
-      <c r="Y6" s="33"/>
-      <c r="Z6" s="33"/>
-      <c r="AA6" s="33"/>
-      <c r="AB6" s="33"/>
-      <c r="AC6" s="33"/>
-      <c r="AD6" s="33"/>
-      <c r="AE6" s="34"/>
-      <c r="AF6" s="32" t="s">
+      <c r="W6" s="48"/>
+      <c r="X6" s="48"/>
+      <c r="Y6" s="48"/>
+      <c r="Z6" s="48"/>
+      <c r="AA6" s="48"/>
+      <c r="AB6" s="48"/>
+      <c r="AC6" s="48"/>
+      <c r="AD6" s="48"/>
+      <c r="AE6" s="49"/>
+      <c r="AF6" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="AG6" s="33"/>
-      <c r="AH6" s="33"/>
-      <c r="AI6" s="33"/>
-      <c r="AJ6" s="33"/>
-      <c r="AK6" s="33"/>
-      <c r="AL6" s="33"/>
-      <c r="AM6" s="33"/>
-      <c r="AN6" s="33"/>
-      <c r="AO6" s="34"/>
-      <c r="AP6" s="32" t="s">
+      <c r="AG6" s="48"/>
+      <c r="AH6" s="48"/>
+      <c r="AI6" s="48"/>
+      <c r="AJ6" s="48"/>
+      <c r="AK6" s="48"/>
+      <c r="AL6" s="48"/>
+      <c r="AM6" s="48"/>
+      <c r="AN6" s="48"/>
+      <c r="AO6" s="49"/>
+      <c r="AP6" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="AQ6" s="33"/>
-      <c r="AR6" s="33"/>
-      <c r="AS6" s="33"/>
-      <c r="AT6" s="33"/>
-      <c r="AU6" s="33"/>
-      <c r="AV6" s="33"/>
-      <c r="AW6" s="33"/>
-      <c r="AX6" s="33"/>
-      <c r="AY6" s="34"/>
-      <c r="AZ6" s="32" t="s">
+      <c r="AQ6" s="48"/>
+      <c r="AR6" s="48"/>
+      <c r="AS6" s="48"/>
+      <c r="AT6" s="48"/>
+      <c r="AU6" s="48"/>
+      <c r="AV6" s="48"/>
+      <c r="AW6" s="48"/>
+      <c r="AX6" s="48"/>
+      <c r="AY6" s="49"/>
+      <c r="AZ6" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="BA6" s="33"/>
-      <c r="BB6" s="33"/>
-      <c r="BC6" s="33"/>
-      <c r="BD6" s="33"/>
-      <c r="BE6" s="33"/>
-      <c r="BF6" s="33"/>
-      <c r="BG6" s="33"/>
-      <c r="BH6" s="33"/>
-      <c r="BI6" s="34"/>
+      <c r="BA6" s="48"/>
+      <c r="BB6" s="48"/>
+      <c r="BC6" s="48"/>
+      <c r="BD6" s="48"/>
+      <c r="BE6" s="48"/>
+      <c r="BF6" s="48"/>
+      <c r="BG6" s="48"/>
+      <c r="BH6" s="48"/>
+      <c r="BI6" s="49"/>
     </row>
     <row r="7" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -1597,18 +1597,18 @@
       <c r="A8" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="AZ8" s="39" t="s">
+      <c r="AZ8" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="BA8" s="40"/>
-      <c r="BB8" s="40"/>
-      <c r="BC8" s="40"/>
-      <c r="BD8" s="40"/>
-      <c r="BE8" s="40"/>
-      <c r="BF8" s="40"/>
-      <c r="BG8" s="40"/>
-      <c r="BH8" s="40"/>
-      <c r="BI8" s="41"/>
+      <c r="BA8" s="42"/>
+      <c r="BB8" s="42"/>
+      <c r="BC8" s="42"/>
+      <c r="BD8" s="42"/>
+      <c r="BE8" s="42"/>
+      <c r="BF8" s="42"/>
+      <c r="BG8" s="42"/>
+      <c r="BH8" s="42"/>
+      <c r="BI8" s="43"/>
     </row>
     <row r="9" spans="1:61" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -2351,8 +2351,8 @@
       <c r="AG20" s="7"/>
       <c r="AH20" s="7"/>
       <c r="AI20" s="10"/>
-      <c r="AJ20" s="7"/>
-      <c r="AK20" s="7"/>
+      <c r="AJ20" s="10"/>
+      <c r="AK20" s="10"/>
       <c r="AL20" s="7"/>
       <c r="AM20" s="7"/>
       <c r="AN20" s="7"/>
@@ -2479,8 +2479,8 @@
       <c r="AG22" s="10"/>
       <c r="AH22" s="10"/>
       <c r="AI22" s="7"/>
-      <c r="AJ22" s="7"/>
-      <c r="AK22" s="7"/>
+      <c r="AJ22" s="10"/>
+      <c r="AK22" s="10"/>
       <c r="AL22" s="7"/>
       <c r="AM22" s="7"/>
       <c r="AN22" s="7"/>
@@ -3273,7 +3273,7 @@
       <c r="BI34" s="7"/>
     </row>
     <row r="35" spans="1:61" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="44" t="s">
+      <c r="A35" s="39" t="s">
         <v>40</v>
       </c>
       <c r="B35" s="5"/>
@@ -3338,7 +3338,7 @@
       <c r="BI35" s="24"/>
     </row>
     <row r="36" spans="1:61" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="45"/>
+      <c r="A36" s="40"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
@@ -5546,11 +5546,35 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="AZ6:BI6"/>
+    <mergeCell ref="L5:U5"/>
+    <mergeCell ref="V5:AE5"/>
+    <mergeCell ref="AF5:AO5"/>
+    <mergeCell ref="AP5:AY5"/>
+    <mergeCell ref="AZ5:BI5"/>
+    <mergeCell ref="B6:K6"/>
+    <mergeCell ref="L6:U6"/>
+    <mergeCell ref="V6:AE6"/>
+    <mergeCell ref="AF6:AO6"/>
+    <mergeCell ref="AP6:AY6"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="AZ8:BI8"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A61:A62"/>
     <mergeCell ref="A63:A64"/>
@@ -5567,35 +5591,11 @@
     <mergeCell ref="A33:A34"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="AZ8:BI8"/>
-    <mergeCell ref="B5:K5"/>
-    <mergeCell ref="AZ6:BI6"/>
-    <mergeCell ref="L5:U5"/>
-    <mergeCell ref="V5:AE5"/>
-    <mergeCell ref="AF5:AO5"/>
-    <mergeCell ref="AP5:AY5"/>
-    <mergeCell ref="AZ5:BI5"/>
-    <mergeCell ref="B6:K6"/>
-    <mergeCell ref="L6:U6"/>
-    <mergeCell ref="V6:AE6"/>
-    <mergeCell ref="AF6:AO6"/>
-    <mergeCell ref="AP6:AY6"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5615,12 +5615,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="47"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -5639,29 +5639,29 @@
       <c r="Q1" s="17"/>
     </row>
     <row r="2" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="48" t="s">
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="49"/>
+      <c r="G2" s="32"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="48" t="s">
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="49"/>
+      <c r="G3" s="32"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:52" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -5669,222 +5669,222 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="42" t="s">
+      <c r="F4" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="43"/>
+      <c r="G4" s="34"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="44">
         <v>8</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="29">
+      <c r="C5" s="45"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="44">
         <v>9</v>
       </c>
-      <c r="F5" s="30"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="50" t="s">
+      <c r="F5" s="45"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="51"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="29">
+      <c r="I5" s="54"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="44">
         <v>11</v>
       </c>
-      <c r="L5" s="30"/>
-      <c r="M5" s="31"/>
-      <c r="N5" s="50" t="s">
+      <c r="L5" s="45"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="51"/>
-      <c r="P5" s="52"/>
-      <c r="Q5" s="29">
+      <c r="O5" s="54"/>
+      <c r="P5" s="55"/>
+      <c r="Q5" s="44">
         <v>13</v>
       </c>
-      <c r="R5" s="30"/>
-      <c r="S5" s="31"/>
-      <c r="T5" s="29">
+      <c r="R5" s="45"/>
+      <c r="S5" s="46"/>
+      <c r="T5" s="44">
         <v>14</v>
       </c>
-      <c r="U5" s="30"/>
-      <c r="V5" s="31"/>
-      <c r="W5" s="59">
+      <c r="U5" s="45"/>
+      <c r="V5" s="46"/>
+      <c r="W5" s="56">
         <v>15</v>
       </c>
-      <c r="X5" s="60"/>
-      <c r="Y5" s="61"/>
-      <c r="Z5" s="29">
+      <c r="X5" s="57"/>
+      <c r="Y5" s="58"/>
+      <c r="Z5" s="44">
         <v>16</v>
       </c>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="31"/>
-      <c r="AC5" s="29">
+      <c r="AA5" s="45"/>
+      <c r="AB5" s="46"/>
+      <c r="AC5" s="44">
         <v>17</v>
       </c>
-      <c r="AD5" s="30"/>
-      <c r="AE5" s="31"/>
-      <c r="AF5" s="29">
+      <c r="AD5" s="45"/>
+      <c r="AE5" s="46"/>
+      <c r="AF5" s="44">
         <v>18</v>
       </c>
-      <c r="AG5" s="30"/>
-      <c r="AH5" s="31"/>
-      <c r="AI5" s="29">
+      <c r="AG5" s="45"/>
+      <c r="AH5" s="46"/>
+      <c r="AI5" s="44">
         <v>19</v>
       </c>
-      <c r="AJ5" s="30"/>
-      <c r="AK5" s="31"/>
-      <c r="AL5" s="29">
+      <c r="AJ5" s="45"/>
+      <c r="AK5" s="46"/>
+      <c r="AL5" s="44">
         <v>20</v>
       </c>
-      <c r="AM5" s="30"/>
-      <c r="AN5" s="31"/>
-      <c r="AO5" s="29">
+      <c r="AM5" s="45"/>
+      <c r="AN5" s="46"/>
+      <c r="AO5" s="44">
         <v>21</v>
       </c>
-      <c r="AP5" s="30"/>
-      <c r="AQ5" s="31"/>
-      <c r="AR5" s="29">
+      <c r="AP5" s="45"/>
+      <c r="AQ5" s="46"/>
+      <c r="AR5" s="44">
         <v>22</v>
       </c>
-      <c r="AS5" s="30"/>
-      <c r="AT5" s="31"/>
-      <c r="AU5" s="29">
+      <c r="AS5" s="45"/>
+      <c r="AT5" s="46"/>
+      <c r="AU5" s="44">
         <v>23</v>
       </c>
-      <c r="AV5" s="30"/>
-      <c r="AW5" s="31"/>
-      <c r="AX5" s="50">
+      <c r="AV5" s="45"/>
+      <c r="AW5" s="46"/>
+      <c r="AX5" s="53">
         <v>24</v>
       </c>
-      <c r="AY5" s="51"/>
-      <c r="AZ5" s="52"/>
+      <c r="AY5" s="54"/>
+      <c r="AZ5" s="55"/>
     </row>
     <row r="6" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="47">
         <v>16.02</v>
       </c>
-      <c r="C6" s="34"/>
+      <c r="C6" s="49"/>
       <c r="D6" s="2">
         <v>19.02</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="47">
         <v>23.02</v>
       </c>
-      <c r="F6" s="34"/>
+      <c r="F6" s="49"/>
       <c r="G6" s="2">
         <v>26.02</v>
       </c>
-      <c r="H6" s="32">
+      <c r="H6" s="47">
         <v>2.0299999999999998</v>
       </c>
-      <c r="I6" s="34"/>
+      <c r="I6" s="49"/>
       <c r="J6" s="2">
         <v>5.03</v>
       </c>
-      <c r="K6" s="32">
+      <c r="K6" s="47">
         <v>9.0299999999999994</v>
       </c>
-      <c r="L6" s="34"/>
+      <c r="L6" s="49"/>
       <c r="M6" s="2">
         <v>12.03</v>
       </c>
-      <c r="N6" s="32">
+      <c r="N6" s="47">
         <v>16.03</v>
       </c>
-      <c r="O6" s="34"/>
+      <c r="O6" s="49"/>
       <c r="P6" s="2">
         <v>19.03</v>
       </c>
-      <c r="Q6" s="32">
+      <c r="Q6" s="47">
         <v>23.03</v>
       </c>
-      <c r="R6" s="34"/>
+      <c r="R6" s="49"/>
       <c r="S6" s="2">
         <v>26.03</v>
       </c>
-      <c r="T6" s="32">
+      <c r="T6" s="47">
         <v>30.03</v>
       </c>
-      <c r="U6" s="34"/>
+      <c r="U6" s="49"/>
       <c r="V6" s="2">
         <v>2.04</v>
       </c>
-      <c r="W6" s="62">
+      <c r="W6" s="59">
         <v>6.04</v>
       </c>
-      <c r="X6" s="63"/>
+      <c r="X6" s="60"/>
       <c r="Y6" s="3">
         <v>9.0399999999999991</v>
       </c>
-      <c r="Z6" s="32">
+      <c r="Z6" s="47">
         <v>13.04</v>
       </c>
-      <c r="AA6" s="34"/>
+      <c r="AA6" s="49"/>
       <c r="AB6" s="2">
         <v>16.04</v>
       </c>
-      <c r="AC6" s="32">
+      <c r="AC6" s="47">
         <v>20.04</v>
       </c>
-      <c r="AD6" s="34"/>
+      <c r="AD6" s="49"/>
       <c r="AE6" s="2">
         <v>23.04</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="47">
         <v>27.04</v>
       </c>
-      <c r="AG6" s="34"/>
+      <c r="AG6" s="49"/>
       <c r="AH6" s="2">
         <v>30.04</v>
       </c>
-      <c r="AI6" s="32">
+      <c r="AI6" s="47">
         <v>4.05</v>
       </c>
-      <c r="AJ6" s="34"/>
+      <c r="AJ6" s="49"/>
       <c r="AK6" s="2">
         <v>7.05</v>
       </c>
-      <c r="AL6" s="32">
+      <c r="AL6" s="47">
         <v>11.05</v>
       </c>
-      <c r="AM6" s="34"/>
+      <c r="AM6" s="49"/>
       <c r="AN6" s="2">
         <v>14.05</v>
       </c>
-      <c r="AO6" s="32">
+      <c r="AO6" s="47">
         <v>18.05</v>
       </c>
-      <c r="AP6" s="34"/>
+      <c r="AP6" s="49"/>
       <c r="AQ6" s="2">
         <v>21.05</v>
       </c>
-      <c r="AR6" s="32">
+      <c r="AR6" s="47">
         <v>25.05</v>
       </c>
-      <c r="AS6" s="34"/>
+      <c r="AS6" s="49"/>
       <c r="AT6" s="2">
         <v>28.05</v>
       </c>
-      <c r="AU6" s="32">
+      <c r="AU6" s="47">
         <v>1.06</v>
       </c>
-      <c r="AV6" s="34"/>
+      <c r="AV6" s="49"/>
       <c r="AW6" s="2">
         <v>4.0599999999999996</v>
       </c>
-      <c r="AX6" s="32">
+      <c r="AX6" s="47">
         <v>8.06</v>
       </c>
-      <c r="AY6" s="34"/>
+      <c r="AY6" s="49"/>
       <c r="AZ6" s="2">
         <v>11.06</v>
       </c>
@@ -6051,32 +6051,32 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="39" t="s">
+      <c r="H8" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="40"/>
-      <c r="J8" s="41"/>
-      <c r="K8" s="64" t="s">
+      <c r="I8" s="42"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="61" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="65"/>
-      <c r="M8" s="66"/>
-      <c r="N8" s="53" t="s">
+      <c r="L8" s="62"/>
+      <c r="M8" s="63"/>
+      <c r="N8" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="O8" s="54"/>
-      <c r="P8" s="55"/>
+      <c r="O8" s="65"/>
+      <c r="P8" s="66"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
-      <c r="W8" s="56" t="s">
+      <c r="W8" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="X8" s="57"/>
-      <c r="Y8" s="58"/>
+      <c r="X8" s="51"/>
+      <c r="Y8" s="52"/>
       <c r="Z8" s="4"/>
       <c r="AA8" s="4"/>
       <c r="AB8" s="4"/>
@@ -6101,11 +6101,11 @@
       <c r="AU8" s="4"/>
       <c r="AV8" s="4"/>
       <c r="AW8" s="4"/>
-      <c r="AX8" s="39" t="s">
+      <c r="AX8" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="AY8" s="40"/>
-      <c r="AZ8" s="41"/>
+      <c r="AY8" s="42"/>
+      <c r="AZ8" s="43"/>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -7976,7 +7976,7 @@
       <c r="AZ42" s="7"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A43" s="44" t="s">
+      <c r="A43" s="39" t="s">
         <v>40</v>
       </c>
       <c r="B43" s="5"/>
@@ -8032,7 +8032,7 @@
       <c r="AZ43" s="5"/>
     </row>
     <row r="44" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="45"/>
+      <c r="A44" s="40"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -8197,6 +8197,54 @@
     </row>
   </sheetData>
   <mergeCells count="64">
+    <mergeCell ref="AU5:AW5"/>
+    <mergeCell ref="AU6:AV6"/>
+    <mergeCell ref="AX5:AZ5"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="AO6:AP6"/>
+    <mergeCell ref="AR5:AT5"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="AC6:AD6"/>
+    <mergeCell ref="AF5:AH5"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H6:I6"/>
     <mergeCell ref="AX8:AZ8"/>
     <mergeCell ref="W8:Y8"/>
     <mergeCell ref="K5:M5"/>
@@ -8213,54 +8261,6 @@
     <mergeCell ref="Z6:AA6"/>
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="AC5:AE5"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="AC6:AD6"/>
-    <mergeCell ref="AF5:AH5"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="AU5:AW5"/>
-    <mergeCell ref="AU6:AV6"/>
-    <mergeCell ref="AX5:AZ5"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="AO5:AQ5"/>
-    <mergeCell ref="AO6:AP6"/>
-    <mergeCell ref="AR5:AT5"/>
-    <mergeCell ref="AR6:AS6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
updated redaction of mechanical design, modelisation
</commit_message>
<xml_diff>
--- a/A_Documentation/Planning.xlsx
+++ b/A_Documentation/Planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\Documents\Repositories\Self-Balancing-Bot\A_Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E713F251-6174-40CF-86AB-4ABD5C2131B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B3886E-2700-444B-9391-5D4DF243E620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -664,51 +664,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -727,14 +682,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -744,6 +735,24 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -767,15 +776,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1205,12 +1205,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="30"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="47"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -1218,29 +1218,29 @@
       <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="31" t="s">
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="32"/>
+      <c r="G2" s="49"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31" t="s">
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="32"/>
+      <c r="G3" s="49"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:61" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -1248,165 +1248,165 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="33" t="s">
+      <c r="F4" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="34"/>
+      <c r="G4" s="43"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="44">
+      <c r="B5" s="29">
         <v>25</v>
       </c>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="45"/>
-      <c r="I5" s="45"/>
-      <c r="J5" s="45"/>
-      <c r="K5" s="46"/>
-      <c r="L5" s="44">
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="29">
         <v>26</v>
       </c>
-      <c r="M5" s="45"/>
-      <c r="N5" s="45"/>
-      <c r="O5" s="45"/>
-      <c r="P5" s="45"/>
-      <c r="Q5" s="45"/>
-      <c r="R5" s="45"/>
-      <c r="S5" s="45"/>
-      <c r="T5" s="45"/>
-      <c r="U5" s="46"/>
-      <c r="V5" s="44">
+      <c r="M5" s="30"/>
+      <c r="N5" s="30"/>
+      <c r="O5" s="30"/>
+      <c r="P5" s="30"/>
+      <c r="Q5" s="30"/>
+      <c r="R5" s="30"/>
+      <c r="S5" s="30"/>
+      <c r="T5" s="30"/>
+      <c r="U5" s="31"/>
+      <c r="V5" s="29">
         <v>27</v>
       </c>
-      <c r="W5" s="45"/>
-      <c r="X5" s="45"/>
-      <c r="Y5" s="45"/>
-      <c r="Z5" s="45"/>
-      <c r="AA5" s="45"/>
-      <c r="AB5" s="45"/>
-      <c r="AC5" s="45"/>
-      <c r="AD5" s="45"/>
-      <c r="AE5" s="46"/>
-      <c r="AF5" s="44">
+      <c r="W5" s="30"/>
+      <c r="X5" s="30"/>
+      <c r="Y5" s="30"/>
+      <c r="Z5" s="30"/>
+      <c r="AA5" s="30"/>
+      <c r="AB5" s="30"/>
+      <c r="AC5" s="30"/>
+      <c r="AD5" s="30"/>
+      <c r="AE5" s="31"/>
+      <c r="AF5" s="29">
         <v>28</v>
       </c>
-      <c r="AG5" s="45"/>
-      <c r="AH5" s="45"/>
-      <c r="AI5" s="45"/>
-      <c r="AJ5" s="45"/>
-      <c r="AK5" s="45"/>
-      <c r="AL5" s="45"/>
-      <c r="AM5" s="45"/>
-      <c r="AN5" s="45"/>
-      <c r="AO5" s="46"/>
-      <c r="AP5" s="44">
+      <c r="AG5" s="30"/>
+      <c r="AH5" s="30"/>
+      <c r="AI5" s="30"/>
+      <c r="AJ5" s="30"/>
+      <c r="AK5" s="30"/>
+      <c r="AL5" s="30"/>
+      <c r="AM5" s="30"/>
+      <c r="AN5" s="30"/>
+      <c r="AO5" s="31"/>
+      <c r="AP5" s="29">
         <v>29</v>
       </c>
-      <c r="AQ5" s="45"/>
-      <c r="AR5" s="45"/>
-      <c r="AS5" s="45"/>
-      <c r="AT5" s="45"/>
-      <c r="AU5" s="45"/>
-      <c r="AV5" s="45"/>
-      <c r="AW5" s="45"/>
-      <c r="AX5" s="45"/>
-      <c r="AY5" s="46"/>
-      <c r="AZ5" s="44">
+      <c r="AQ5" s="30"/>
+      <c r="AR5" s="30"/>
+      <c r="AS5" s="30"/>
+      <c r="AT5" s="30"/>
+      <c r="AU5" s="30"/>
+      <c r="AV5" s="30"/>
+      <c r="AW5" s="30"/>
+      <c r="AX5" s="30"/>
+      <c r="AY5" s="31"/>
+      <c r="AZ5" s="29">
         <v>30</v>
       </c>
-      <c r="BA5" s="45"/>
-      <c r="BB5" s="45"/>
-      <c r="BC5" s="45"/>
-      <c r="BD5" s="45"/>
-      <c r="BE5" s="45"/>
-      <c r="BF5" s="45"/>
-      <c r="BG5" s="45"/>
-      <c r="BH5" s="45"/>
-      <c r="BI5" s="46"/>
+      <c r="BA5" s="30"/>
+      <c r="BB5" s="30"/>
+      <c r="BC5" s="30"/>
+      <c r="BD5" s="30"/>
+      <c r="BE5" s="30"/>
+      <c r="BF5" s="30"/>
+      <c r="BG5" s="30"/>
+      <c r="BH5" s="30"/>
+      <c r="BI5" s="31"/>
     </row>
     <row r="6" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="49"/>
-      <c r="L6" s="47" t="s">
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="34"/>
+      <c r="L6" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="48"/>
-      <c r="N6" s="48"/>
-      <c r="O6" s="48"/>
-      <c r="P6" s="48"/>
-      <c r="Q6" s="48"/>
-      <c r="R6" s="48"/>
-      <c r="S6" s="48"/>
-      <c r="T6" s="48"/>
-      <c r="U6" s="49"/>
-      <c r="V6" s="47" t="s">
+      <c r="M6" s="33"/>
+      <c r="N6" s="33"/>
+      <c r="O6" s="33"/>
+      <c r="P6" s="33"/>
+      <c r="Q6" s="33"/>
+      <c r="R6" s="33"/>
+      <c r="S6" s="33"/>
+      <c r="T6" s="33"/>
+      <c r="U6" s="34"/>
+      <c r="V6" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="W6" s="48"/>
-      <c r="X6" s="48"/>
-      <c r="Y6" s="48"/>
-      <c r="Z6" s="48"/>
-      <c r="AA6" s="48"/>
-      <c r="AB6" s="48"/>
-      <c r="AC6" s="48"/>
-      <c r="AD6" s="48"/>
-      <c r="AE6" s="49"/>
-      <c r="AF6" s="47" t="s">
+      <c r="W6" s="33"/>
+      <c r="X6" s="33"/>
+      <c r="Y6" s="33"/>
+      <c r="Z6" s="33"/>
+      <c r="AA6" s="33"/>
+      <c r="AB6" s="33"/>
+      <c r="AC6" s="33"/>
+      <c r="AD6" s="33"/>
+      <c r="AE6" s="34"/>
+      <c r="AF6" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="AG6" s="48"/>
-      <c r="AH6" s="48"/>
-      <c r="AI6" s="48"/>
-      <c r="AJ6" s="48"/>
-      <c r="AK6" s="48"/>
-      <c r="AL6" s="48"/>
-      <c r="AM6" s="48"/>
-      <c r="AN6" s="48"/>
-      <c r="AO6" s="49"/>
-      <c r="AP6" s="47" t="s">
+      <c r="AG6" s="33"/>
+      <c r="AH6" s="33"/>
+      <c r="AI6" s="33"/>
+      <c r="AJ6" s="33"/>
+      <c r="AK6" s="33"/>
+      <c r="AL6" s="33"/>
+      <c r="AM6" s="33"/>
+      <c r="AN6" s="33"/>
+      <c r="AO6" s="34"/>
+      <c r="AP6" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="AQ6" s="48"/>
-      <c r="AR6" s="48"/>
-      <c r="AS6" s="48"/>
-      <c r="AT6" s="48"/>
-      <c r="AU6" s="48"/>
-      <c r="AV6" s="48"/>
-      <c r="AW6" s="48"/>
-      <c r="AX6" s="48"/>
-      <c r="AY6" s="49"/>
-      <c r="AZ6" s="47" t="s">
+      <c r="AQ6" s="33"/>
+      <c r="AR6" s="33"/>
+      <c r="AS6" s="33"/>
+      <c r="AT6" s="33"/>
+      <c r="AU6" s="33"/>
+      <c r="AV6" s="33"/>
+      <c r="AW6" s="33"/>
+      <c r="AX6" s="33"/>
+      <c r="AY6" s="34"/>
+      <c r="AZ6" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="BA6" s="48"/>
-      <c r="BB6" s="48"/>
-      <c r="BC6" s="48"/>
-      <c r="BD6" s="48"/>
-      <c r="BE6" s="48"/>
-      <c r="BF6" s="48"/>
-      <c r="BG6" s="48"/>
-      <c r="BH6" s="48"/>
-      <c r="BI6" s="49"/>
+      <c r="BA6" s="33"/>
+      <c r="BB6" s="33"/>
+      <c r="BC6" s="33"/>
+      <c r="BD6" s="33"/>
+      <c r="BE6" s="33"/>
+      <c r="BF6" s="33"/>
+      <c r="BG6" s="33"/>
+      <c r="BH6" s="33"/>
+      <c r="BI6" s="34"/>
     </row>
     <row r="7" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -1597,18 +1597,18 @@
       <c r="A8" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="AZ8" s="41" t="s">
+      <c r="AZ8" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="BA8" s="42"/>
-      <c r="BB8" s="42"/>
-      <c r="BC8" s="42"/>
-      <c r="BD8" s="42"/>
-      <c r="BE8" s="42"/>
-      <c r="BF8" s="42"/>
-      <c r="BG8" s="42"/>
-      <c r="BH8" s="42"/>
-      <c r="BI8" s="43"/>
+      <c r="BA8" s="40"/>
+      <c r="BB8" s="40"/>
+      <c r="BC8" s="40"/>
+      <c r="BD8" s="40"/>
+      <c r="BE8" s="40"/>
+      <c r="BF8" s="40"/>
+      <c r="BG8" s="40"/>
+      <c r="BH8" s="40"/>
+      <c r="BI8" s="41"/>
     </row>
     <row r="9" spans="1:61" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -2353,10 +2353,10 @@
       <c r="AI20" s="10"/>
       <c r="AJ20" s="10"/>
       <c r="AK20" s="10"/>
-      <c r="AL20" s="7"/>
-      <c r="AM20" s="7"/>
-      <c r="AN20" s="7"/>
-      <c r="AO20" s="7"/>
+      <c r="AL20" s="10"/>
+      <c r="AM20" s="10"/>
+      <c r="AN20" s="10"/>
+      <c r="AO20" s="10"/>
       <c r="AP20" s="7"/>
       <c r="AQ20" s="7"/>
       <c r="AR20" s="7"/>
@@ -2481,10 +2481,10 @@
       <c r="AI22" s="7"/>
       <c r="AJ22" s="10"/>
       <c r="AK22" s="10"/>
-      <c r="AL22" s="7"/>
-      <c r="AM22" s="7"/>
-      <c r="AN22" s="7"/>
-      <c r="AO22" s="7"/>
+      <c r="AL22" s="10"/>
+      <c r="AM22" s="10"/>
+      <c r="AN22" s="10"/>
+      <c r="AO22" s="10"/>
       <c r="AP22" s="7"/>
       <c r="AQ22" s="7"/>
       <c r="AR22" s="7"/>
@@ -2599,7 +2599,7 @@
       <c r="Y24" s="7"/>
       <c r="Z24" s="7"/>
       <c r="AA24" s="7"/>
-      <c r="AB24" s="7"/>
+      <c r="AB24" s="10"/>
       <c r="AC24" s="7"/>
       <c r="AD24" s="7"/>
       <c r="AE24" s="7"/>
@@ -3273,7 +3273,7 @@
       <c r="BI34" s="7"/>
     </row>
     <row r="35" spans="1:61" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="39" t="s">
+      <c r="A35" s="44" t="s">
         <v>40</v>
       </c>
       <c r="B35" s="5"/>
@@ -3338,7 +3338,7 @@
       <c r="BI35" s="24"/>
     </row>
     <row r="36" spans="1:61" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="40"/>
+      <c r="A36" s="45"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
@@ -5546,35 +5546,11 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="B5:K5"/>
-    <mergeCell ref="AZ6:BI6"/>
-    <mergeCell ref="L5:U5"/>
-    <mergeCell ref="V5:AE5"/>
-    <mergeCell ref="AF5:AO5"/>
-    <mergeCell ref="AP5:AY5"/>
-    <mergeCell ref="AZ5:BI5"/>
-    <mergeCell ref="B6:K6"/>
-    <mergeCell ref="L6:U6"/>
-    <mergeCell ref="V6:AE6"/>
-    <mergeCell ref="AF6:AO6"/>
-    <mergeCell ref="AP6:AY6"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="AZ8:BI8"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A61:A62"/>
     <mergeCell ref="A63:A64"/>
@@ -5591,11 +5567,35 @@
     <mergeCell ref="A33:A34"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="AZ8:BI8"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="AZ6:BI6"/>
+    <mergeCell ref="L5:U5"/>
+    <mergeCell ref="V5:AE5"/>
+    <mergeCell ref="AF5:AO5"/>
+    <mergeCell ref="AP5:AY5"/>
+    <mergeCell ref="AZ5:BI5"/>
+    <mergeCell ref="B6:K6"/>
+    <mergeCell ref="L6:U6"/>
+    <mergeCell ref="V6:AE6"/>
+    <mergeCell ref="AF6:AO6"/>
+    <mergeCell ref="AP6:AY6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5615,12 +5615,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="30"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="47"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -5639,29 +5639,29 @@
       <c r="Q1" s="17"/>
     </row>
     <row r="2" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="31" t="s">
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="32"/>
+      <c r="G2" s="49"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31" t="s">
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="32"/>
+      <c r="G3" s="49"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:52" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -5669,222 +5669,222 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="33" t="s">
+      <c r="F4" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="34"/>
+      <c r="G4" s="43"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="44">
+      <c r="B5" s="29">
         <v>8</v>
       </c>
-      <c r="C5" s="45"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="44">
+      <c r="C5" s="30"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="29">
         <v>9</v>
       </c>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
-      <c r="H5" s="53" t="s">
+      <c r="F5" s="30"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="54"/>
-      <c r="J5" s="55"/>
-      <c r="K5" s="44">
+      <c r="I5" s="51"/>
+      <c r="J5" s="52"/>
+      <c r="K5" s="29">
         <v>11</v>
       </c>
-      <c r="L5" s="45"/>
-      <c r="M5" s="46"/>
-      <c r="N5" s="53" t="s">
+      <c r="L5" s="30"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="54"/>
-      <c r="P5" s="55"/>
-      <c r="Q5" s="44">
+      <c r="O5" s="51"/>
+      <c r="P5" s="52"/>
+      <c r="Q5" s="29">
         <v>13</v>
       </c>
-      <c r="R5" s="45"/>
-      <c r="S5" s="46"/>
-      <c r="T5" s="44">
+      <c r="R5" s="30"/>
+      <c r="S5" s="31"/>
+      <c r="T5" s="29">
         <v>14</v>
       </c>
-      <c r="U5" s="45"/>
-      <c r="V5" s="46"/>
-      <c r="W5" s="56">
+      <c r="U5" s="30"/>
+      <c r="V5" s="31"/>
+      <c r="W5" s="59">
         <v>15</v>
       </c>
-      <c r="X5" s="57"/>
-      <c r="Y5" s="58"/>
-      <c r="Z5" s="44">
+      <c r="X5" s="60"/>
+      <c r="Y5" s="61"/>
+      <c r="Z5" s="29">
         <v>16</v>
       </c>
-      <c r="AA5" s="45"/>
-      <c r="AB5" s="46"/>
-      <c r="AC5" s="44">
+      <c r="AA5" s="30"/>
+      <c r="AB5" s="31"/>
+      <c r="AC5" s="29">
         <v>17</v>
       </c>
-      <c r="AD5" s="45"/>
-      <c r="AE5" s="46"/>
-      <c r="AF5" s="44">
+      <c r="AD5" s="30"/>
+      <c r="AE5" s="31"/>
+      <c r="AF5" s="29">
         <v>18</v>
       </c>
-      <c r="AG5" s="45"/>
-      <c r="AH5" s="46"/>
-      <c r="AI5" s="44">
+      <c r="AG5" s="30"/>
+      <c r="AH5" s="31"/>
+      <c r="AI5" s="29">
         <v>19</v>
       </c>
-      <c r="AJ5" s="45"/>
-      <c r="AK5" s="46"/>
-      <c r="AL5" s="44">
+      <c r="AJ5" s="30"/>
+      <c r="AK5" s="31"/>
+      <c r="AL5" s="29">
         <v>20</v>
       </c>
-      <c r="AM5" s="45"/>
-      <c r="AN5" s="46"/>
-      <c r="AO5" s="44">
+      <c r="AM5" s="30"/>
+      <c r="AN5" s="31"/>
+      <c r="AO5" s="29">
         <v>21</v>
       </c>
-      <c r="AP5" s="45"/>
-      <c r="AQ5" s="46"/>
-      <c r="AR5" s="44">
+      <c r="AP5" s="30"/>
+      <c r="AQ5" s="31"/>
+      <c r="AR5" s="29">
         <v>22</v>
       </c>
-      <c r="AS5" s="45"/>
-      <c r="AT5" s="46"/>
-      <c r="AU5" s="44">
+      <c r="AS5" s="30"/>
+      <c r="AT5" s="31"/>
+      <c r="AU5" s="29">
         <v>23</v>
       </c>
-      <c r="AV5" s="45"/>
-      <c r="AW5" s="46"/>
-      <c r="AX5" s="53">
+      <c r="AV5" s="30"/>
+      <c r="AW5" s="31"/>
+      <c r="AX5" s="50">
         <v>24</v>
       </c>
-      <c r="AY5" s="54"/>
-      <c r="AZ5" s="55"/>
+      <c r="AY5" s="51"/>
+      <c r="AZ5" s="52"/>
     </row>
     <row r="6" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="47">
+      <c r="B6" s="32">
         <v>16.02</v>
       </c>
-      <c r="C6" s="49"/>
+      <c r="C6" s="34"/>
       <c r="D6" s="2">
         <v>19.02</v>
       </c>
-      <c r="E6" s="47">
+      <c r="E6" s="32">
         <v>23.02</v>
       </c>
-      <c r="F6" s="49"/>
+      <c r="F6" s="34"/>
       <c r="G6" s="2">
         <v>26.02</v>
       </c>
-      <c r="H6" s="47">
+      <c r="H6" s="32">
         <v>2.0299999999999998</v>
       </c>
-      <c r="I6" s="49"/>
+      <c r="I6" s="34"/>
       <c r="J6" s="2">
         <v>5.03</v>
       </c>
-      <c r="K6" s="47">
+      <c r="K6" s="32">
         <v>9.0299999999999994</v>
       </c>
-      <c r="L6" s="49"/>
+      <c r="L6" s="34"/>
       <c r="M6" s="2">
         <v>12.03</v>
       </c>
-      <c r="N6" s="47">
+      <c r="N6" s="32">
         <v>16.03</v>
       </c>
-      <c r="O6" s="49"/>
+      <c r="O6" s="34"/>
       <c r="P6" s="2">
         <v>19.03</v>
       </c>
-      <c r="Q6" s="47">
+      <c r="Q6" s="32">
         <v>23.03</v>
       </c>
-      <c r="R6" s="49"/>
+      <c r="R6" s="34"/>
       <c r="S6" s="2">
         <v>26.03</v>
       </c>
-      <c r="T6" s="47">
+      <c r="T6" s="32">
         <v>30.03</v>
       </c>
-      <c r="U6" s="49"/>
+      <c r="U6" s="34"/>
       <c r="V6" s="2">
         <v>2.04</v>
       </c>
-      <c r="W6" s="59">
+      <c r="W6" s="62">
         <v>6.04</v>
       </c>
-      <c r="X6" s="60"/>
+      <c r="X6" s="63"/>
       <c r="Y6" s="3">
         <v>9.0399999999999991</v>
       </c>
-      <c r="Z6" s="47">
+      <c r="Z6" s="32">
         <v>13.04</v>
       </c>
-      <c r="AA6" s="49"/>
+      <c r="AA6" s="34"/>
       <c r="AB6" s="2">
         <v>16.04</v>
       </c>
-      <c r="AC6" s="47">
+      <c r="AC6" s="32">
         <v>20.04</v>
       </c>
-      <c r="AD6" s="49"/>
+      <c r="AD6" s="34"/>
       <c r="AE6" s="2">
         <v>23.04</v>
       </c>
-      <c r="AF6" s="47">
+      <c r="AF6" s="32">
         <v>27.04</v>
       </c>
-      <c r="AG6" s="49"/>
+      <c r="AG6" s="34"/>
       <c r="AH6" s="2">
         <v>30.04</v>
       </c>
-      <c r="AI6" s="47">
+      <c r="AI6" s="32">
         <v>4.05</v>
       </c>
-      <c r="AJ6" s="49"/>
+      <c r="AJ6" s="34"/>
       <c r="AK6" s="2">
         <v>7.05</v>
       </c>
-      <c r="AL6" s="47">
+      <c r="AL6" s="32">
         <v>11.05</v>
       </c>
-      <c r="AM6" s="49"/>
+      <c r="AM6" s="34"/>
       <c r="AN6" s="2">
         <v>14.05</v>
       </c>
-      <c r="AO6" s="47">
+      <c r="AO6" s="32">
         <v>18.05</v>
       </c>
-      <c r="AP6" s="49"/>
+      <c r="AP6" s="34"/>
       <c r="AQ6" s="2">
         <v>21.05</v>
       </c>
-      <c r="AR6" s="47">
+      <c r="AR6" s="32">
         <v>25.05</v>
       </c>
-      <c r="AS6" s="49"/>
+      <c r="AS6" s="34"/>
       <c r="AT6" s="2">
         <v>28.05</v>
       </c>
-      <c r="AU6" s="47">
+      <c r="AU6" s="32">
         <v>1.06</v>
       </c>
-      <c r="AV6" s="49"/>
+      <c r="AV6" s="34"/>
       <c r="AW6" s="2">
         <v>4.0599999999999996</v>
       </c>
-      <c r="AX6" s="47">
+      <c r="AX6" s="32">
         <v>8.06</v>
       </c>
-      <c r="AY6" s="49"/>
+      <c r="AY6" s="34"/>
       <c r="AZ6" s="2">
         <v>11.06</v>
       </c>
@@ -6051,32 +6051,32 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="41" t="s">
+      <c r="H8" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="42"/>
-      <c r="J8" s="43"/>
-      <c r="K8" s="61" t="s">
+      <c r="I8" s="40"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="64" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="62"/>
-      <c r="M8" s="63"/>
-      <c r="N8" s="64" t="s">
+      <c r="L8" s="65"/>
+      <c r="M8" s="66"/>
+      <c r="N8" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="O8" s="65"/>
-      <c r="P8" s="66"/>
+      <c r="O8" s="54"/>
+      <c r="P8" s="55"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
-      <c r="W8" s="50" t="s">
+      <c r="W8" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="X8" s="51"/>
-      <c r="Y8" s="52"/>
+      <c r="X8" s="57"/>
+      <c r="Y8" s="58"/>
       <c r="Z8" s="4"/>
       <c r="AA8" s="4"/>
       <c r="AB8" s="4"/>
@@ -6101,11 +6101,11 @@
       <c r="AU8" s="4"/>
       <c r="AV8" s="4"/>
       <c r="AW8" s="4"/>
-      <c r="AX8" s="41" t="s">
+      <c r="AX8" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="AY8" s="42"/>
-      <c r="AZ8" s="43"/>
+      <c r="AY8" s="40"/>
+      <c r="AZ8" s="41"/>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -7976,7 +7976,7 @@
       <c r="AZ42" s="7"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A43" s="39" t="s">
+      <c r="A43" s="44" t="s">
         <v>40</v>
       </c>
       <c r="B43" s="5"/>
@@ -8032,7 +8032,7 @@
       <c r="AZ43" s="5"/>
     </row>
     <row r="44" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="40"/>
+      <c r="A44" s="45"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -8197,54 +8197,6 @@
     </row>
   </sheetData>
   <mergeCells count="64">
-    <mergeCell ref="AU5:AW5"/>
-    <mergeCell ref="AU6:AV6"/>
-    <mergeCell ref="AX5:AZ5"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="AO5:AQ5"/>
-    <mergeCell ref="AO6:AP6"/>
-    <mergeCell ref="AR5:AT5"/>
-    <mergeCell ref="AR6:AS6"/>
-    <mergeCell ref="AC6:AD6"/>
-    <mergeCell ref="AF5:AH5"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H6:I6"/>
     <mergeCell ref="AX8:AZ8"/>
     <mergeCell ref="W8:Y8"/>
     <mergeCell ref="K5:M5"/>
@@ -8261,6 +8213,54 @@
     <mergeCell ref="Z6:AA6"/>
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="AC5:AE5"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="AC6:AD6"/>
+    <mergeCell ref="AF5:AH5"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="AU5:AW5"/>
+    <mergeCell ref="AU6:AV6"/>
+    <mergeCell ref="AX5:AZ5"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="AO6:AP6"/>
+    <mergeCell ref="AR5:AT5"/>
+    <mergeCell ref="AR6:AS6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Matlab modifications, modelisation redaction
</commit_message>
<xml_diff>
--- a/A_Documentation/Planning.xlsx
+++ b/A_Documentation/Planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\Documents\Repositories\Self-Balancing-Bot\A_Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B3886E-2700-444B-9391-5D4DF243E620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B890D827-1B25-45A1-9A85-2881293A8F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2357,10 +2357,10 @@
       <c r="AM20" s="10"/>
       <c r="AN20" s="10"/>
       <c r="AO20" s="10"/>
-      <c r="AP20" s="7"/>
-      <c r="AQ20" s="7"/>
-      <c r="AR20" s="7"/>
-      <c r="AS20" s="7"/>
+      <c r="AP20" s="10"/>
+      <c r="AQ20" s="10"/>
+      <c r="AR20" s="10"/>
+      <c r="AS20" s="10"/>
       <c r="AT20" s="7"/>
       <c r="AU20" s="7"/>
       <c r="AV20" s="7"/>
@@ -2613,10 +2613,10 @@
       <c r="AM24" s="7"/>
       <c r="AN24" s="7"/>
       <c r="AO24" s="7"/>
-      <c r="AP24" s="7"/>
-      <c r="AQ24" s="7"/>
-      <c r="AR24" s="7"/>
-      <c r="AS24" s="7"/>
+      <c r="AP24" s="10"/>
+      <c r="AQ24" s="10"/>
+      <c r="AR24" s="10"/>
+      <c r="AS24" s="10"/>
       <c r="AT24" s="7"/>
       <c r="AU24" s="7"/>
       <c r="AV24" s="7"/>

</xml_diff>

<commit_message>
Finished analysis, conclusion started
</commit_message>
<xml_diff>
--- a/A_Documentation/Planning.xlsx
+++ b/A_Documentation/Planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\Documents\Repositories\Self-Balancing-Bot\A_Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B890D827-1B25-45A1-9A85-2881293A8F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EDCBC39-3643-44D6-818B-4F1B13D8AAA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -664,6 +664,51 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -682,50 +727,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -735,24 +744,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -776,6 +767,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1205,12 +1205,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="47"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -1218,29 +1218,29 @@
       <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="48" t="s">
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="49"/>
+      <c r="G2" s="32"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="48" t="s">
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="49"/>
+      <c r="G3" s="32"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:61" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -1248,165 +1248,165 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="42" t="s">
+      <c r="F4" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="43"/>
+      <c r="G4" s="34"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="44">
         <v>25</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="31"/>
-      <c r="L5" s="29">
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="46"/>
+      <c r="L5" s="44">
         <v>26</v>
       </c>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
-      <c r="P5" s="30"/>
-      <c r="Q5" s="30"/>
-      <c r="R5" s="30"/>
-      <c r="S5" s="30"/>
-      <c r="T5" s="30"/>
-      <c r="U5" s="31"/>
-      <c r="V5" s="29">
+      <c r="M5" s="45"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="45"/>
+      <c r="P5" s="45"/>
+      <c r="Q5" s="45"/>
+      <c r="R5" s="45"/>
+      <c r="S5" s="45"/>
+      <c r="T5" s="45"/>
+      <c r="U5" s="46"/>
+      <c r="V5" s="44">
         <v>27</v>
       </c>
-      <c r="W5" s="30"/>
-      <c r="X5" s="30"/>
-      <c r="Y5" s="30"/>
-      <c r="Z5" s="30"/>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="30"/>
-      <c r="AC5" s="30"/>
-      <c r="AD5" s="30"/>
-      <c r="AE5" s="31"/>
-      <c r="AF5" s="29">
+      <c r="W5" s="45"/>
+      <c r="X5" s="45"/>
+      <c r="Y5" s="45"/>
+      <c r="Z5" s="45"/>
+      <c r="AA5" s="45"/>
+      <c r="AB5" s="45"/>
+      <c r="AC5" s="45"/>
+      <c r="AD5" s="45"/>
+      <c r="AE5" s="46"/>
+      <c r="AF5" s="44">
         <v>28</v>
       </c>
-      <c r="AG5" s="30"/>
-      <c r="AH5" s="30"/>
-      <c r="AI5" s="30"/>
-      <c r="AJ5" s="30"/>
-      <c r="AK5" s="30"/>
-      <c r="AL5" s="30"/>
-      <c r="AM5" s="30"/>
-      <c r="AN5" s="30"/>
-      <c r="AO5" s="31"/>
-      <c r="AP5" s="29">
+      <c r="AG5" s="45"/>
+      <c r="AH5" s="45"/>
+      <c r="AI5" s="45"/>
+      <c r="AJ5" s="45"/>
+      <c r="AK5" s="45"/>
+      <c r="AL5" s="45"/>
+      <c r="AM5" s="45"/>
+      <c r="AN5" s="45"/>
+      <c r="AO5" s="46"/>
+      <c r="AP5" s="44">
         <v>29</v>
       </c>
-      <c r="AQ5" s="30"/>
-      <c r="AR5" s="30"/>
-      <c r="AS5" s="30"/>
-      <c r="AT5" s="30"/>
-      <c r="AU5" s="30"/>
-      <c r="AV5" s="30"/>
-      <c r="AW5" s="30"/>
-      <c r="AX5" s="30"/>
-      <c r="AY5" s="31"/>
-      <c r="AZ5" s="29">
+      <c r="AQ5" s="45"/>
+      <c r="AR5" s="45"/>
+      <c r="AS5" s="45"/>
+      <c r="AT5" s="45"/>
+      <c r="AU5" s="45"/>
+      <c r="AV5" s="45"/>
+      <c r="AW5" s="45"/>
+      <c r="AX5" s="45"/>
+      <c r="AY5" s="46"/>
+      <c r="AZ5" s="44">
         <v>30</v>
       </c>
-      <c r="BA5" s="30"/>
-      <c r="BB5" s="30"/>
-      <c r="BC5" s="30"/>
-      <c r="BD5" s="30"/>
-      <c r="BE5" s="30"/>
-      <c r="BF5" s="30"/>
-      <c r="BG5" s="30"/>
-      <c r="BH5" s="30"/>
-      <c r="BI5" s="31"/>
+      <c r="BA5" s="45"/>
+      <c r="BB5" s="45"/>
+      <c r="BC5" s="45"/>
+      <c r="BD5" s="45"/>
+      <c r="BE5" s="45"/>
+      <c r="BF5" s="45"/>
+      <c r="BG5" s="45"/>
+      <c r="BH5" s="45"/>
+      <c r="BI5" s="46"/>
     </row>
     <row r="6" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="33"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="32" t="s">
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="33"/>
-      <c r="N6" s="33"/>
-      <c r="O6" s="33"/>
-      <c r="P6" s="33"/>
-      <c r="Q6" s="33"/>
-      <c r="R6" s="33"/>
-      <c r="S6" s="33"/>
-      <c r="T6" s="33"/>
-      <c r="U6" s="34"/>
-      <c r="V6" s="32" t="s">
+      <c r="M6" s="48"/>
+      <c r="N6" s="48"/>
+      <c r="O6" s="48"/>
+      <c r="P6" s="48"/>
+      <c r="Q6" s="48"/>
+      <c r="R6" s="48"/>
+      <c r="S6" s="48"/>
+      <c r="T6" s="48"/>
+      <c r="U6" s="49"/>
+      <c r="V6" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="W6" s="33"/>
-      <c r="X6" s="33"/>
-      <c r="Y6" s="33"/>
-      <c r="Z6" s="33"/>
-      <c r="AA6" s="33"/>
-      <c r="AB6" s="33"/>
-      <c r="AC6" s="33"/>
-      <c r="AD6" s="33"/>
-      <c r="AE6" s="34"/>
-      <c r="AF6" s="32" t="s">
+      <c r="W6" s="48"/>
+      <c r="X6" s="48"/>
+      <c r="Y6" s="48"/>
+      <c r="Z6" s="48"/>
+      <c r="AA6" s="48"/>
+      <c r="AB6" s="48"/>
+      <c r="AC6" s="48"/>
+      <c r="AD6" s="48"/>
+      <c r="AE6" s="49"/>
+      <c r="AF6" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="AG6" s="33"/>
-      <c r="AH6" s="33"/>
-      <c r="AI6" s="33"/>
-      <c r="AJ6" s="33"/>
-      <c r="AK6" s="33"/>
-      <c r="AL6" s="33"/>
-      <c r="AM6" s="33"/>
-      <c r="AN6" s="33"/>
-      <c r="AO6" s="34"/>
-      <c r="AP6" s="32" t="s">
+      <c r="AG6" s="48"/>
+      <c r="AH6" s="48"/>
+      <c r="AI6" s="48"/>
+      <c r="AJ6" s="48"/>
+      <c r="AK6" s="48"/>
+      <c r="AL6" s="48"/>
+      <c r="AM6" s="48"/>
+      <c r="AN6" s="48"/>
+      <c r="AO6" s="49"/>
+      <c r="AP6" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="AQ6" s="33"/>
-      <c r="AR6" s="33"/>
-      <c r="AS6" s="33"/>
-      <c r="AT6" s="33"/>
-      <c r="AU6" s="33"/>
-      <c r="AV6" s="33"/>
-      <c r="AW6" s="33"/>
-      <c r="AX6" s="33"/>
-      <c r="AY6" s="34"/>
-      <c r="AZ6" s="32" t="s">
+      <c r="AQ6" s="48"/>
+      <c r="AR6" s="48"/>
+      <c r="AS6" s="48"/>
+      <c r="AT6" s="48"/>
+      <c r="AU6" s="48"/>
+      <c r="AV6" s="48"/>
+      <c r="AW6" s="48"/>
+      <c r="AX6" s="48"/>
+      <c r="AY6" s="49"/>
+      <c r="AZ6" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="BA6" s="33"/>
-      <c r="BB6" s="33"/>
-      <c r="BC6" s="33"/>
-      <c r="BD6" s="33"/>
-      <c r="BE6" s="33"/>
-      <c r="BF6" s="33"/>
-      <c r="BG6" s="33"/>
-      <c r="BH6" s="33"/>
-      <c r="BI6" s="34"/>
+      <c r="BA6" s="48"/>
+      <c r="BB6" s="48"/>
+      <c r="BC6" s="48"/>
+      <c r="BD6" s="48"/>
+      <c r="BE6" s="48"/>
+      <c r="BF6" s="48"/>
+      <c r="BG6" s="48"/>
+      <c r="BH6" s="48"/>
+      <c r="BI6" s="49"/>
     </row>
     <row r="7" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -1597,18 +1597,18 @@
       <c r="A8" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="AZ8" s="39" t="s">
+      <c r="AZ8" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="BA8" s="40"/>
-      <c r="BB8" s="40"/>
-      <c r="BC8" s="40"/>
-      <c r="BD8" s="40"/>
-      <c r="BE8" s="40"/>
-      <c r="BF8" s="40"/>
-      <c r="BG8" s="40"/>
-      <c r="BH8" s="40"/>
-      <c r="BI8" s="41"/>
+      <c r="BA8" s="42"/>
+      <c r="BB8" s="42"/>
+      <c r="BC8" s="42"/>
+      <c r="BD8" s="42"/>
+      <c r="BE8" s="42"/>
+      <c r="BF8" s="42"/>
+      <c r="BG8" s="42"/>
+      <c r="BH8" s="42"/>
+      <c r="BI8" s="43"/>
     </row>
     <row r="9" spans="1:61" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -2617,16 +2617,16 @@
       <c r="AQ24" s="10"/>
       <c r="AR24" s="10"/>
       <c r="AS24" s="10"/>
-      <c r="AT24" s="7"/>
-      <c r="AU24" s="7"/>
-      <c r="AV24" s="7"/>
-      <c r="AW24" s="7"/>
-      <c r="AX24" s="7"/>
-      <c r="AY24" s="7"/>
-      <c r="AZ24" s="7"/>
-      <c r="BA24" s="7"/>
-      <c r="BB24" s="7"/>
-      <c r="BC24" s="7"/>
+      <c r="AT24" s="10"/>
+      <c r="AU24" s="10"/>
+      <c r="AV24" s="10"/>
+      <c r="AW24" s="10"/>
+      <c r="AX24" s="10"/>
+      <c r="AY24" s="10"/>
+      <c r="AZ24" s="10"/>
+      <c r="BA24" s="10"/>
+      <c r="BB24" s="10"/>
+      <c r="BC24" s="10"/>
       <c r="BD24" s="7"/>
       <c r="BE24" s="7"/>
       <c r="BF24" s="7"/>
@@ -2880,9 +2880,9 @@
       <c r="AX28" s="7"/>
       <c r="AY28" s="7"/>
       <c r="AZ28" s="7"/>
-      <c r="BA28" s="7"/>
-      <c r="BB28" s="7"/>
-      <c r="BC28" s="7"/>
+      <c r="BA28" s="10"/>
+      <c r="BB28" s="10"/>
+      <c r="BC28" s="10"/>
       <c r="BD28" s="7"/>
       <c r="BE28" s="7"/>
       <c r="BF28" s="7"/>
@@ -3273,7 +3273,7 @@
       <c r="BI34" s="7"/>
     </row>
     <row r="35" spans="1:61" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="44" t="s">
+      <c r="A35" s="39" t="s">
         <v>40</v>
       </c>
       <c r="B35" s="5"/>
@@ -3338,7 +3338,7 @@
       <c r="BI35" s="24"/>
     </row>
     <row r="36" spans="1:61" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="45"/>
+      <c r="A36" s="40"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
@@ -5546,11 +5546,35 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="AZ6:BI6"/>
+    <mergeCell ref="L5:U5"/>
+    <mergeCell ref="V5:AE5"/>
+    <mergeCell ref="AF5:AO5"/>
+    <mergeCell ref="AP5:AY5"/>
+    <mergeCell ref="AZ5:BI5"/>
+    <mergeCell ref="B6:K6"/>
+    <mergeCell ref="L6:U6"/>
+    <mergeCell ref="V6:AE6"/>
+    <mergeCell ref="AF6:AO6"/>
+    <mergeCell ref="AP6:AY6"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="AZ8:BI8"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A61:A62"/>
     <mergeCell ref="A63:A64"/>
@@ -5567,35 +5591,11 @@
     <mergeCell ref="A33:A34"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="AZ8:BI8"/>
-    <mergeCell ref="B5:K5"/>
-    <mergeCell ref="AZ6:BI6"/>
-    <mergeCell ref="L5:U5"/>
-    <mergeCell ref="V5:AE5"/>
-    <mergeCell ref="AF5:AO5"/>
-    <mergeCell ref="AP5:AY5"/>
-    <mergeCell ref="AZ5:BI5"/>
-    <mergeCell ref="B6:K6"/>
-    <mergeCell ref="L6:U6"/>
-    <mergeCell ref="V6:AE6"/>
-    <mergeCell ref="AF6:AO6"/>
-    <mergeCell ref="AP6:AY6"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5615,12 +5615,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="47"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -5639,29 +5639,29 @@
       <c r="Q1" s="17"/>
     </row>
     <row r="2" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="48" t="s">
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="49"/>
+      <c r="G2" s="32"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="48" t="s">
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="49"/>
+      <c r="G3" s="32"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:52" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -5669,222 +5669,222 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="42" t="s">
+      <c r="F4" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="43"/>
+      <c r="G4" s="34"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="44">
         <v>8</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="29">
+      <c r="C5" s="45"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="44">
         <v>9</v>
       </c>
-      <c r="F5" s="30"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="50" t="s">
+      <c r="F5" s="45"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="51"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="29">
+      <c r="I5" s="54"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="44">
         <v>11</v>
       </c>
-      <c r="L5" s="30"/>
-      <c r="M5" s="31"/>
-      <c r="N5" s="50" t="s">
+      <c r="L5" s="45"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="51"/>
-      <c r="P5" s="52"/>
-      <c r="Q5" s="29">
+      <c r="O5" s="54"/>
+      <c r="P5" s="55"/>
+      <c r="Q5" s="44">
         <v>13</v>
       </c>
-      <c r="R5" s="30"/>
-      <c r="S5" s="31"/>
-      <c r="T5" s="29">
+      <c r="R5" s="45"/>
+      <c r="S5" s="46"/>
+      <c r="T5" s="44">
         <v>14</v>
       </c>
-      <c r="U5" s="30"/>
-      <c r="V5" s="31"/>
-      <c r="W5" s="59">
+      <c r="U5" s="45"/>
+      <c r="V5" s="46"/>
+      <c r="W5" s="56">
         <v>15</v>
       </c>
-      <c r="X5" s="60"/>
-      <c r="Y5" s="61"/>
-      <c r="Z5" s="29">
+      <c r="X5" s="57"/>
+      <c r="Y5" s="58"/>
+      <c r="Z5" s="44">
         <v>16</v>
       </c>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="31"/>
-      <c r="AC5" s="29">
+      <c r="AA5" s="45"/>
+      <c r="AB5" s="46"/>
+      <c r="AC5" s="44">
         <v>17</v>
       </c>
-      <c r="AD5" s="30"/>
-      <c r="AE5" s="31"/>
-      <c r="AF5" s="29">
+      <c r="AD5" s="45"/>
+      <c r="AE5" s="46"/>
+      <c r="AF5" s="44">
         <v>18</v>
       </c>
-      <c r="AG5" s="30"/>
-      <c r="AH5" s="31"/>
-      <c r="AI5" s="29">
+      <c r="AG5" s="45"/>
+      <c r="AH5" s="46"/>
+      <c r="AI5" s="44">
         <v>19</v>
       </c>
-      <c r="AJ5" s="30"/>
-      <c r="AK5" s="31"/>
-      <c r="AL5" s="29">
+      <c r="AJ5" s="45"/>
+      <c r="AK5" s="46"/>
+      <c r="AL5" s="44">
         <v>20</v>
       </c>
-      <c r="AM5" s="30"/>
-      <c r="AN5" s="31"/>
-      <c r="AO5" s="29">
+      <c r="AM5" s="45"/>
+      <c r="AN5" s="46"/>
+      <c r="AO5" s="44">
         <v>21</v>
       </c>
-      <c r="AP5" s="30"/>
-      <c r="AQ5" s="31"/>
-      <c r="AR5" s="29">
+      <c r="AP5" s="45"/>
+      <c r="AQ5" s="46"/>
+      <c r="AR5" s="44">
         <v>22</v>
       </c>
-      <c r="AS5" s="30"/>
-      <c r="AT5" s="31"/>
-      <c r="AU5" s="29">
+      <c r="AS5" s="45"/>
+      <c r="AT5" s="46"/>
+      <c r="AU5" s="44">
         <v>23</v>
       </c>
-      <c r="AV5" s="30"/>
-      <c r="AW5" s="31"/>
-      <c r="AX5" s="50">
+      <c r="AV5" s="45"/>
+      <c r="AW5" s="46"/>
+      <c r="AX5" s="53">
         <v>24</v>
       </c>
-      <c r="AY5" s="51"/>
-      <c r="AZ5" s="52"/>
+      <c r="AY5" s="54"/>
+      <c r="AZ5" s="55"/>
     </row>
     <row r="6" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="47">
         <v>16.02</v>
       </c>
-      <c r="C6" s="34"/>
+      <c r="C6" s="49"/>
       <c r="D6" s="2">
         <v>19.02</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="47">
         <v>23.02</v>
       </c>
-      <c r="F6" s="34"/>
+      <c r="F6" s="49"/>
       <c r="G6" s="2">
         <v>26.02</v>
       </c>
-      <c r="H6" s="32">
+      <c r="H6" s="47">
         <v>2.0299999999999998</v>
       </c>
-      <c r="I6" s="34"/>
+      <c r="I6" s="49"/>
       <c r="J6" s="2">
         <v>5.03</v>
       </c>
-      <c r="K6" s="32">
+      <c r="K6" s="47">
         <v>9.0299999999999994</v>
       </c>
-      <c r="L6" s="34"/>
+      <c r="L6" s="49"/>
       <c r="M6" s="2">
         <v>12.03</v>
       </c>
-      <c r="N6" s="32">
+      <c r="N6" s="47">
         <v>16.03</v>
       </c>
-      <c r="O6" s="34"/>
+      <c r="O6" s="49"/>
       <c r="P6" s="2">
         <v>19.03</v>
       </c>
-      <c r="Q6" s="32">
+      <c r="Q6" s="47">
         <v>23.03</v>
       </c>
-      <c r="R6" s="34"/>
+      <c r="R6" s="49"/>
       <c r="S6" s="2">
         <v>26.03</v>
       </c>
-      <c r="T6" s="32">
+      <c r="T6" s="47">
         <v>30.03</v>
       </c>
-      <c r="U6" s="34"/>
+      <c r="U6" s="49"/>
       <c r="V6" s="2">
         <v>2.04</v>
       </c>
-      <c r="W6" s="62">
+      <c r="W6" s="59">
         <v>6.04</v>
       </c>
-      <c r="X6" s="63"/>
+      <c r="X6" s="60"/>
       <c r="Y6" s="3">
         <v>9.0399999999999991</v>
       </c>
-      <c r="Z6" s="32">
+      <c r="Z6" s="47">
         <v>13.04</v>
       </c>
-      <c r="AA6" s="34"/>
+      <c r="AA6" s="49"/>
       <c r="AB6" s="2">
         <v>16.04</v>
       </c>
-      <c r="AC6" s="32">
+      <c r="AC6" s="47">
         <v>20.04</v>
       </c>
-      <c r="AD6" s="34"/>
+      <c r="AD6" s="49"/>
       <c r="AE6" s="2">
         <v>23.04</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="47">
         <v>27.04</v>
       </c>
-      <c r="AG6" s="34"/>
+      <c r="AG6" s="49"/>
       <c r="AH6" s="2">
         <v>30.04</v>
       </c>
-      <c r="AI6" s="32">
+      <c r="AI6" s="47">
         <v>4.05</v>
       </c>
-      <c r="AJ6" s="34"/>
+      <c r="AJ6" s="49"/>
       <c r="AK6" s="2">
         <v>7.05</v>
       </c>
-      <c r="AL6" s="32">
+      <c r="AL6" s="47">
         <v>11.05</v>
       </c>
-      <c r="AM6" s="34"/>
+      <c r="AM6" s="49"/>
       <c r="AN6" s="2">
         <v>14.05</v>
       </c>
-      <c r="AO6" s="32">
+      <c r="AO6" s="47">
         <v>18.05</v>
       </c>
-      <c r="AP6" s="34"/>
+      <c r="AP6" s="49"/>
       <c r="AQ6" s="2">
         <v>21.05</v>
       </c>
-      <c r="AR6" s="32">
+      <c r="AR6" s="47">
         <v>25.05</v>
       </c>
-      <c r="AS6" s="34"/>
+      <c r="AS6" s="49"/>
       <c r="AT6" s="2">
         <v>28.05</v>
       </c>
-      <c r="AU6" s="32">
+      <c r="AU6" s="47">
         <v>1.06</v>
       </c>
-      <c r="AV6" s="34"/>
+      <c r="AV6" s="49"/>
       <c r="AW6" s="2">
         <v>4.0599999999999996</v>
       </c>
-      <c r="AX6" s="32">
+      <c r="AX6" s="47">
         <v>8.06</v>
       </c>
-      <c r="AY6" s="34"/>
+      <c r="AY6" s="49"/>
       <c r="AZ6" s="2">
         <v>11.06</v>
       </c>
@@ -6051,32 +6051,32 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="39" t="s">
+      <c r="H8" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="40"/>
-      <c r="J8" s="41"/>
-      <c r="K8" s="64" t="s">
+      <c r="I8" s="42"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="61" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="65"/>
-      <c r="M8" s="66"/>
-      <c r="N8" s="53" t="s">
+      <c r="L8" s="62"/>
+      <c r="M8" s="63"/>
+      <c r="N8" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="O8" s="54"/>
-      <c r="P8" s="55"/>
+      <c r="O8" s="65"/>
+      <c r="P8" s="66"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
-      <c r="W8" s="56" t="s">
+      <c r="W8" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="X8" s="57"/>
-      <c r="Y8" s="58"/>
+      <c r="X8" s="51"/>
+      <c r="Y8" s="52"/>
       <c r="Z8" s="4"/>
       <c r="AA8" s="4"/>
       <c r="AB8" s="4"/>
@@ -6101,11 +6101,11 @@
       <c r="AU8" s="4"/>
       <c r="AV8" s="4"/>
       <c r="AW8" s="4"/>
-      <c r="AX8" s="39" t="s">
+      <c r="AX8" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="AY8" s="40"/>
-      <c r="AZ8" s="41"/>
+      <c r="AY8" s="42"/>
+      <c r="AZ8" s="43"/>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -7976,7 +7976,7 @@
       <c r="AZ42" s="7"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A43" s="44" t="s">
+      <c r="A43" s="39" t="s">
         <v>40</v>
       </c>
       <c r="B43" s="5"/>
@@ -8032,7 +8032,7 @@
       <c r="AZ43" s="5"/>
     </row>
     <row r="44" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="45"/>
+      <c r="A44" s="40"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -8197,6 +8197,54 @@
     </row>
   </sheetData>
   <mergeCells count="64">
+    <mergeCell ref="AU5:AW5"/>
+    <mergeCell ref="AU6:AV6"/>
+    <mergeCell ref="AX5:AZ5"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="AO6:AP6"/>
+    <mergeCell ref="AR5:AT5"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="AC6:AD6"/>
+    <mergeCell ref="AF5:AH5"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H6:I6"/>
     <mergeCell ref="AX8:AZ8"/>
     <mergeCell ref="W8:Y8"/>
     <mergeCell ref="K5:M5"/>
@@ -8213,54 +8261,6 @@
     <mergeCell ref="Z6:AA6"/>
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="AC5:AE5"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="AC6:AD6"/>
-    <mergeCell ref="AF5:AH5"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="AU5:AW5"/>
-    <mergeCell ref="AU6:AV6"/>
-    <mergeCell ref="AX5:AZ5"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="AO5:AQ5"/>
-    <mergeCell ref="AO6:AP6"/>
-    <mergeCell ref="AR5:AT5"/>
-    <mergeCell ref="AR6:AS6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Measurement of PLA wheels, updated planning, BOM, redaction of conclusion
</commit_message>
<xml_diff>
--- a/A_Documentation/Planning.xlsx
+++ b/A_Documentation/Planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\Documents\Repositories\Self-Balancing-Bot\A_Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EDCBC39-3643-44D6-818B-4F1B13D8AAA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CDDD4BF-0D29-4813-B8B6-959F0D1E91F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -664,51 +664,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -727,14 +682,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -744,6 +735,24 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -767,15 +776,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1205,12 +1205,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="30"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="47"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -1218,29 +1218,29 @@
       <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="31" t="s">
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="32"/>
+      <c r="G2" s="49"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31" t="s">
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="32"/>
+      <c r="G3" s="49"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:61" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -1248,165 +1248,165 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="33" t="s">
+      <c r="F4" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="34"/>
+      <c r="G4" s="43"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="44">
+      <c r="B5" s="29">
         <v>25</v>
       </c>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="45"/>
-      <c r="I5" s="45"/>
-      <c r="J5" s="45"/>
-      <c r="K5" s="46"/>
-      <c r="L5" s="44">
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="29">
         <v>26</v>
       </c>
-      <c r="M5" s="45"/>
-      <c r="N5" s="45"/>
-      <c r="O5" s="45"/>
-      <c r="P5" s="45"/>
-      <c r="Q5" s="45"/>
-      <c r="R5" s="45"/>
-      <c r="S5" s="45"/>
-      <c r="T5" s="45"/>
-      <c r="U5" s="46"/>
-      <c r="V5" s="44">
+      <c r="M5" s="30"/>
+      <c r="N5" s="30"/>
+      <c r="O5" s="30"/>
+      <c r="P5" s="30"/>
+      <c r="Q5" s="30"/>
+      <c r="R5" s="30"/>
+      <c r="S5" s="30"/>
+      <c r="T5" s="30"/>
+      <c r="U5" s="31"/>
+      <c r="V5" s="29">
         <v>27</v>
       </c>
-      <c r="W5" s="45"/>
-      <c r="X5" s="45"/>
-      <c r="Y5" s="45"/>
-      <c r="Z5" s="45"/>
-      <c r="AA5" s="45"/>
-      <c r="AB5" s="45"/>
-      <c r="AC5" s="45"/>
-      <c r="AD5" s="45"/>
-      <c r="AE5" s="46"/>
-      <c r="AF5" s="44">
+      <c r="W5" s="30"/>
+      <c r="X5" s="30"/>
+      <c r="Y5" s="30"/>
+      <c r="Z5" s="30"/>
+      <c r="AA5" s="30"/>
+      <c r="AB5" s="30"/>
+      <c r="AC5" s="30"/>
+      <c r="AD5" s="30"/>
+      <c r="AE5" s="31"/>
+      <c r="AF5" s="29">
         <v>28</v>
       </c>
-      <c r="AG5" s="45"/>
-      <c r="AH5" s="45"/>
-      <c r="AI5" s="45"/>
-      <c r="AJ5" s="45"/>
-      <c r="AK5" s="45"/>
-      <c r="AL5" s="45"/>
-      <c r="AM5" s="45"/>
-      <c r="AN5" s="45"/>
-      <c r="AO5" s="46"/>
-      <c r="AP5" s="44">
+      <c r="AG5" s="30"/>
+      <c r="AH5" s="30"/>
+      <c r="AI5" s="30"/>
+      <c r="AJ5" s="30"/>
+      <c r="AK5" s="30"/>
+      <c r="AL5" s="30"/>
+      <c r="AM5" s="30"/>
+      <c r="AN5" s="30"/>
+      <c r="AO5" s="31"/>
+      <c r="AP5" s="29">
         <v>29</v>
       </c>
-      <c r="AQ5" s="45"/>
-      <c r="AR5" s="45"/>
-      <c r="AS5" s="45"/>
-      <c r="AT5" s="45"/>
-      <c r="AU5" s="45"/>
-      <c r="AV5" s="45"/>
-      <c r="AW5" s="45"/>
-      <c r="AX5" s="45"/>
-      <c r="AY5" s="46"/>
-      <c r="AZ5" s="44">
+      <c r="AQ5" s="30"/>
+      <c r="AR5" s="30"/>
+      <c r="AS5" s="30"/>
+      <c r="AT5" s="30"/>
+      <c r="AU5" s="30"/>
+      <c r="AV5" s="30"/>
+      <c r="AW5" s="30"/>
+      <c r="AX5" s="30"/>
+      <c r="AY5" s="31"/>
+      <c r="AZ5" s="29">
         <v>30</v>
       </c>
-      <c r="BA5" s="45"/>
-      <c r="BB5" s="45"/>
-      <c r="BC5" s="45"/>
-      <c r="BD5" s="45"/>
-      <c r="BE5" s="45"/>
-      <c r="BF5" s="45"/>
-      <c r="BG5" s="45"/>
-      <c r="BH5" s="45"/>
-      <c r="BI5" s="46"/>
+      <c r="BA5" s="30"/>
+      <c r="BB5" s="30"/>
+      <c r="BC5" s="30"/>
+      <c r="BD5" s="30"/>
+      <c r="BE5" s="30"/>
+      <c r="BF5" s="30"/>
+      <c r="BG5" s="30"/>
+      <c r="BH5" s="30"/>
+      <c r="BI5" s="31"/>
     </row>
     <row r="6" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="49"/>
-      <c r="L6" s="47" t="s">
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="34"/>
+      <c r="L6" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="48"/>
-      <c r="N6" s="48"/>
-      <c r="O6" s="48"/>
-      <c r="P6" s="48"/>
-      <c r="Q6" s="48"/>
-      <c r="R6" s="48"/>
-      <c r="S6" s="48"/>
-      <c r="T6" s="48"/>
-      <c r="U6" s="49"/>
-      <c r="V6" s="47" t="s">
+      <c r="M6" s="33"/>
+      <c r="N6" s="33"/>
+      <c r="O6" s="33"/>
+      <c r="P6" s="33"/>
+      <c r="Q6" s="33"/>
+      <c r="R6" s="33"/>
+      <c r="S6" s="33"/>
+      <c r="T6" s="33"/>
+      <c r="U6" s="34"/>
+      <c r="V6" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="W6" s="48"/>
-      <c r="X6" s="48"/>
-      <c r="Y6" s="48"/>
-      <c r="Z6" s="48"/>
-      <c r="AA6" s="48"/>
-      <c r="AB6" s="48"/>
-      <c r="AC6" s="48"/>
-      <c r="AD6" s="48"/>
-      <c r="AE6" s="49"/>
-      <c r="AF6" s="47" t="s">
+      <c r="W6" s="33"/>
+      <c r="X6" s="33"/>
+      <c r="Y6" s="33"/>
+      <c r="Z6" s="33"/>
+      <c r="AA6" s="33"/>
+      <c r="AB6" s="33"/>
+      <c r="AC6" s="33"/>
+      <c r="AD6" s="33"/>
+      <c r="AE6" s="34"/>
+      <c r="AF6" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="AG6" s="48"/>
-      <c r="AH6" s="48"/>
-      <c r="AI6" s="48"/>
-      <c r="AJ6" s="48"/>
-      <c r="AK6" s="48"/>
-      <c r="AL6" s="48"/>
-      <c r="AM6" s="48"/>
-      <c r="AN6" s="48"/>
-      <c r="AO6" s="49"/>
-      <c r="AP6" s="47" t="s">
+      <c r="AG6" s="33"/>
+      <c r="AH6" s="33"/>
+      <c r="AI6" s="33"/>
+      <c r="AJ6" s="33"/>
+      <c r="AK6" s="33"/>
+      <c r="AL6" s="33"/>
+      <c r="AM6" s="33"/>
+      <c r="AN6" s="33"/>
+      <c r="AO6" s="34"/>
+      <c r="AP6" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="AQ6" s="48"/>
-      <c r="AR6" s="48"/>
-      <c r="AS6" s="48"/>
-      <c r="AT6" s="48"/>
-      <c r="AU6" s="48"/>
-      <c r="AV6" s="48"/>
-      <c r="AW6" s="48"/>
-      <c r="AX6" s="48"/>
-      <c r="AY6" s="49"/>
-      <c r="AZ6" s="47" t="s">
+      <c r="AQ6" s="33"/>
+      <c r="AR6" s="33"/>
+      <c r="AS6" s="33"/>
+      <c r="AT6" s="33"/>
+      <c r="AU6" s="33"/>
+      <c r="AV6" s="33"/>
+      <c r="AW6" s="33"/>
+      <c r="AX6" s="33"/>
+      <c r="AY6" s="34"/>
+      <c r="AZ6" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="BA6" s="48"/>
-      <c r="BB6" s="48"/>
-      <c r="BC6" s="48"/>
-      <c r="BD6" s="48"/>
-      <c r="BE6" s="48"/>
-      <c r="BF6" s="48"/>
-      <c r="BG6" s="48"/>
-      <c r="BH6" s="48"/>
-      <c r="BI6" s="49"/>
+      <c r="BA6" s="33"/>
+      <c r="BB6" s="33"/>
+      <c r="BC6" s="33"/>
+      <c r="BD6" s="33"/>
+      <c r="BE6" s="33"/>
+      <c r="BF6" s="33"/>
+      <c r="BG6" s="33"/>
+      <c r="BH6" s="33"/>
+      <c r="BI6" s="34"/>
     </row>
     <row r="7" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -1597,18 +1597,18 @@
       <c r="A8" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="AZ8" s="41" t="s">
+      <c r="AZ8" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="BA8" s="42"/>
-      <c r="BB8" s="42"/>
-      <c r="BC8" s="42"/>
-      <c r="BD8" s="42"/>
-      <c r="BE8" s="42"/>
-      <c r="BF8" s="42"/>
-      <c r="BG8" s="42"/>
-      <c r="BH8" s="42"/>
-      <c r="BI8" s="43"/>
+      <c r="BA8" s="40"/>
+      <c r="BB8" s="40"/>
+      <c r="BC8" s="40"/>
+      <c r="BD8" s="40"/>
+      <c r="BE8" s="40"/>
+      <c r="BF8" s="40"/>
+      <c r="BG8" s="40"/>
+      <c r="BH8" s="40"/>
+      <c r="BI8" s="41"/>
     </row>
     <row r="9" spans="1:61" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -3010,8 +3010,8 @@
       <c r="AZ30" s="7"/>
       <c r="BA30" s="7"/>
       <c r="BB30" s="7"/>
-      <c r="BC30" s="7"/>
-      <c r="BD30" s="7"/>
+      <c r="BC30" s="10"/>
+      <c r="BD30" s="10"/>
       <c r="BE30" s="7"/>
       <c r="BF30" s="7"/>
       <c r="BG30" s="7"/>
@@ -3273,7 +3273,7 @@
       <c r="BI34" s="7"/>
     </row>
     <row r="35" spans="1:61" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="39" t="s">
+      <c r="A35" s="44" t="s">
         <v>40</v>
       </c>
       <c r="B35" s="5"/>
@@ -3338,7 +3338,7 @@
       <c r="BI35" s="24"/>
     </row>
     <row r="36" spans="1:61" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="40"/>
+      <c r="A36" s="45"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
@@ -5546,35 +5546,11 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="B5:K5"/>
-    <mergeCell ref="AZ6:BI6"/>
-    <mergeCell ref="L5:U5"/>
-    <mergeCell ref="V5:AE5"/>
-    <mergeCell ref="AF5:AO5"/>
-    <mergeCell ref="AP5:AY5"/>
-    <mergeCell ref="AZ5:BI5"/>
-    <mergeCell ref="B6:K6"/>
-    <mergeCell ref="L6:U6"/>
-    <mergeCell ref="V6:AE6"/>
-    <mergeCell ref="AF6:AO6"/>
-    <mergeCell ref="AP6:AY6"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="AZ8:BI8"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A61:A62"/>
     <mergeCell ref="A63:A64"/>
@@ -5591,11 +5567,35 @@
     <mergeCell ref="A33:A34"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="AZ8:BI8"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="AZ6:BI6"/>
+    <mergeCell ref="L5:U5"/>
+    <mergeCell ref="V5:AE5"/>
+    <mergeCell ref="AF5:AO5"/>
+    <mergeCell ref="AP5:AY5"/>
+    <mergeCell ref="AZ5:BI5"/>
+    <mergeCell ref="B6:K6"/>
+    <mergeCell ref="L6:U6"/>
+    <mergeCell ref="V6:AE6"/>
+    <mergeCell ref="AF6:AO6"/>
+    <mergeCell ref="AP6:AY6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5615,12 +5615,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="30"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="47"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -5639,29 +5639,29 @@
       <c r="Q1" s="17"/>
     </row>
     <row r="2" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="31" t="s">
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="32"/>
+      <c r="G2" s="49"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31" t="s">
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="32"/>
+      <c r="G3" s="49"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:52" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -5669,222 +5669,222 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="33" t="s">
+      <c r="F4" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="34"/>
+      <c r="G4" s="43"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="44">
+      <c r="B5" s="29">
         <v>8</v>
       </c>
-      <c r="C5" s="45"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="44">
+      <c r="C5" s="30"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="29">
         <v>9</v>
       </c>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
-      <c r="H5" s="53" t="s">
+      <c r="F5" s="30"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="54"/>
-      <c r="J5" s="55"/>
-      <c r="K5" s="44">
+      <c r="I5" s="51"/>
+      <c r="J5" s="52"/>
+      <c r="K5" s="29">
         <v>11</v>
       </c>
-      <c r="L5" s="45"/>
-      <c r="M5" s="46"/>
-      <c r="N5" s="53" t="s">
+      <c r="L5" s="30"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="54"/>
-      <c r="P5" s="55"/>
-      <c r="Q5" s="44">
+      <c r="O5" s="51"/>
+      <c r="P5" s="52"/>
+      <c r="Q5" s="29">
         <v>13</v>
       </c>
-      <c r="R5" s="45"/>
-      <c r="S5" s="46"/>
-      <c r="T5" s="44">
+      <c r="R5" s="30"/>
+      <c r="S5" s="31"/>
+      <c r="T5" s="29">
         <v>14</v>
       </c>
-      <c r="U5" s="45"/>
-      <c r="V5" s="46"/>
-      <c r="W5" s="56">
+      <c r="U5" s="30"/>
+      <c r="V5" s="31"/>
+      <c r="W5" s="59">
         <v>15</v>
       </c>
-      <c r="X5" s="57"/>
-      <c r="Y5" s="58"/>
-      <c r="Z5" s="44">
+      <c r="X5" s="60"/>
+      <c r="Y5" s="61"/>
+      <c r="Z5" s="29">
         <v>16</v>
       </c>
-      <c r="AA5" s="45"/>
-      <c r="AB5" s="46"/>
-      <c r="AC5" s="44">
+      <c r="AA5" s="30"/>
+      <c r="AB5" s="31"/>
+      <c r="AC5" s="29">
         <v>17</v>
       </c>
-      <c r="AD5" s="45"/>
-      <c r="AE5" s="46"/>
-      <c r="AF5" s="44">
+      <c r="AD5" s="30"/>
+      <c r="AE5" s="31"/>
+      <c r="AF5" s="29">
         <v>18</v>
       </c>
-      <c r="AG5" s="45"/>
-      <c r="AH5" s="46"/>
-      <c r="AI5" s="44">
+      <c r="AG5" s="30"/>
+      <c r="AH5" s="31"/>
+      <c r="AI5" s="29">
         <v>19</v>
       </c>
-      <c r="AJ5" s="45"/>
-      <c r="AK5" s="46"/>
-      <c r="AL5" s="44">
+      <c r="AJ5" s="30"/>
+      <c r="AK5" s="31"/>
+      <c r="AL5" s="29">
         <v>20</v>
       </c>
-      <c r="AM5" s="45"/>
-      <c r="AN5" s="46"/>
-      <c r="AO5" s="44">
+      <c r="AM5" s="30"/>
+      <c r="AN5" s="31"/>
+      <c r="AO5" s="29">
         <v>21</v>
       </c>
-      <c r="AP5" s="45"/>
-      <c r="AQ5" s="46"/>
-      <c r="AR5" s="44">
+      <c r="AP5" s="30"/>
+      <c r="AQ5" s="31"/>
+      <c r="AR5" s="29">
         <v>22</v>
       </c>
-      <c r="AS5" s="45"/>
-      <c r="AT5" s="46"/>
-      <c r="AU5" s="44">
+      <c r="AS5" s="30"/>
+      <c r="AT5" s="31"/>
+      <c r="AU5" s="29">
         <v>23</v>
       </c>
-      <c r="AV5" s="45"/>
-      <c r="AW5" s="46"/>
-      <c r="AX5" s="53">
+      <c r="AV5" s="30"/>
+      <c r="AW5" s="31"/>
+      <c r="AX5" s="50">
         <v>24</v>
       </c>
-      <c r="AY5" s="54"/>
-      <c r="AZ5" s="55"/>
+      <c r="AY5" s="51"/>
+      <c r="AZ5" s="52"/>
     </row>
     <row r="6" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="47">
+      <c r="B6" s="32">
         <v>16.02</v>
       </c>
-      <c r="C6" s="49"/>
+      <c r="C6" s="34"/>
       <c r="D6" s="2">
         <v>19.02</v>
       </c>
-      <c r="E6" s="47">
+      <c r="E6" s="32">
         <v>23.02</v>
       </c>
-      <c r="F6" s="49"/>
+      <c r="F6" s="34"/>
       <c r="G6" s="2">
         <v>26.02</v>
       </c>
-      <c r="H6" s="47">
+      <c r="H6" s="32">
         <v>2.0299999999999998</v>
       </c>
-      <c r="I6" s="49"/>
+      <c r="I6" s="34"/>
       <c r="J6" s="2">
         <v>5.03</v>
       </c>
-      <c r="K6" s="47">
+      <c r="K6" s="32">
         <v>9.0299999999999994</v>
       </c>
-      <c r="L6" s="49"/>
+      <c r="L6" s="34"/>
       <c r="M6" s="2">
         <v>12.03</v>
       </c>
-      <c r="N6" s="47">
+      <c r="N6" s="32">
         <v>16.03</v>
       </c>
-      <c r="O6" s="49"/>
+      <c r="O6" s="34"/>
       <c r="P6" s="2">
         <v>19.03</v>
       </c>
-      <c r="Q6" s="47">
+      <c r="Q6" s="32">
         <v>23.03</v>
       </c>
-      <c r="R6" s="49"/>
+      <c r="R6" s="34"/>
       <c r="S6" s="2">
         <v>26.03</v>
       </c>
-      <c r="T6" s="47">
+      <c r="T6" s="32">
         <v>30.03</v>
       </c>
-      <c r="U6" s="49"/>
+      <c r="U6" s="34"/>
       <c r="V6" s="2">
         <v>2.04</v>
       </c>
-      <c r="W6" s="59">
+      <c r="W6" s="62">
         <v>6.04</v>
       </c>
-      <c r="X6" s="60"/>
+      <c r="X6" s="63"/>
       <c r="Y6" s="3">
         <v>9.0399999999999991</v>
       </c>
-      <c r="Z6" s="47">
+      <c r="Z6" s="32">
         <v>13.04</v>
       </c>
-      <c r="AA6" s="49"/>
+      <c r="AA6" s="34"/>
       <c r="AB6" s="2">
         <v>16.04</v>
       </c>
-      <c r="AC6" s="47">
+      <c r="AC6" s="32">
         <v>20.04</v>
       </c>
-      <c r="AD6" s="49"/>
+      <c r="AD6" s="34"/>
       <c r="AE6" s="2">
         <v>23.04</v>
       </c>
-      <c r="AF6" s="47">
+      <c r="AF6" s="32">
         <v>27.04</v>
       </c>
-      <c r="AG6" s="49"/>
+      <c r="AG6" s="34"/>
       <c r="AH6" s="2">
         <v>30.04</v>
       </c>
-      <c r="AI6" s="47">
+      <c r="AI6" s="32">
         <v>4.05</v>
       </c>
-      <c r="AJ6" s="49"/>
+      <c r="AJ6" s="34"/>
       <c r="AK6" s="2">
         <v>7.05</v>
       </c>
-      <c r="AL6" s="47">
+      <c r="AL6" s="32">
         <v>11.05</v>
       </c>
-      <c r="AM6" s="49"/>
+      <c r="AM6" s="34"/>
       <c r="AN6" s="2">
         <v>14.05</v>
       </c>
-      <c r="AO6" s="47">
+      <c r="AO6" s="32">
         <v>18.05</v>
       </c>
-      <c r="AP6" s="49"/>
+      <c r="AP6" s="34"/>
       <c r="AQ6" s="2">
         <v>21.05</v>
       </c>
-      <c r="AR6" s="47">
+      <c r="AR6" s="32">
         <v>25.05</v>
       </c>
-      <c r="AS6" s="49"/>
+      <c r="AS6" s="34"/>
       <c r="AT6" s="2">
         <v>28.05</v>
       </c>
-      <c r="AU6" s="47">
+      <c r="AU6" s="32">
         <v>1.06</v>
       </c>
-      <c r="AV6" s="49"/>
+      <c r="AV6" s="34"/>
       <c r="AW6" s="2">
         <v>4.0599999999999996</v>
       </c>
-      <c r="AX6" s="47">
+      <c r="AX6" s="32">
         <v>8.06</v>
       </c>
-      <c r="AY6" s="49"/>
+      <c r="AY6" s="34"/>
       <c r="AZ6" s="2">
         <v>11.06</v>
       </c>
@@ -6051,32 +6051,32 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="41" t="s">
+      <c r="H8" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="42"/>
-      <c r="J8" s="43"/>
-      <c r="K8" s="61" t="s">
+      <c r="I8" s="40"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="64" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="62"/>
-      <c r="M8" s="63"/>
-      <c r="N8" s="64" t="s">
+      <c r="L8" s="65"/>
+      <c r="M8" s="66"/>
+      <c r="N8" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="O8" s="65"/>
-      <c r="P8" s="66"/>
+      <c r="O8" s="54"/>
+      <c r="P8" s="55"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
-      <c r="W8" s="50" t="s">
+      <c r="W8" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="X8" s="51"/>
-      <c r="Y8" s="52"/>
+      <c r="X8" s="57"/>
+      <c r="Y8" s="58"/>
       <c r="Z8" s="4"/>
       <c r="AA8" s="4"/>
       <c r="AB8" s="4"/>
@@ -6101,11 +6101,11 @@
       <c r="AU8" s="4"/>
       <c r="AV8" s="4"/>
       <c r="AW8" s="4"/>
-      <c r="AX8" s="41" t="s">
+      <c r="AX8" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="AY8" s="42"/>
-      <c r="AZ8" s="43"/>
+      <c r="AY8" s="40"/>
+      <c r="AZ8" s="41"/>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -7976,7 +7976,7 @@
       <c r="AZ42" s="7"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A43" s="39" t="s">
+      <c r="A43" s="44" t="s">
         <v>40</v>
       </c>
       <c r="B43" s="5"/>
@@ -8032,7 +8032,7 @@
       <c r="AZ43" s="5"/>
     </row>
     <row r="44" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="40"/>
+      <c r="A44" s="45"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -8197,54 +8197,6 @@
     </row>
   </sheetData>
   <mergeCells count="64">
-    <mergeCell ref="AU5:AW5"/>
-    <mergeCell ref="AU6:AV6"/>
-    <mergeCell ref="AX5:AZ5"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="AO5:AQ5"/>
-    <mergeCell ref="AO6:AP6"/>
-    <mergeCell ref="AR5:AT5"/>
-    <mergeCell ref="AR6:AS6"/>
-    <mergeCell ref="AC6:AD6"/>
-    <mergeCell ref="AF5:AH5"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H6:I6"/>
     <mergeCell ref="AX8:AZ8"/>
     <mergeCell ref="W8:Y8"/>
     <mergeCell ref="K5:M5"/>
@@ -8261,6 +8213,54 @@
     <mergeCell ref="Z6:AA6"/>
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="AC5:AE5"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="AC6:AD6"/>
+    <mergeCell ref="AF5:AH5"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="AU5:AW5"/>
+    <mergeCell ref="AU6:AV6"/>
+    <mergeCell ref="AX5:AZ5"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="AO6:AP6"/>
+    <mergeCell ref="AR5:AT5"/>
+    <mergeCell ref="AR6:AS6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added user guide, updated planning
</commit_message>
<xml_diff>
--- a/A_Documentation/Planning.xlsx
+++ b/A_Documentation/Planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\Documents\Repositories\Self-Balancing-Bot\A_Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CDDD4BF-0D29-4813-B8B6-959F0D1E91F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D64602D-35CE-416E-AB7C-95796EC522BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -664,6 +664,51 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -682,50 +727,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -735,24 +744,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -776,6 +767,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1205,12 +1205,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="47"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -1218,29 +1218,29 @@
       <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="48" t="s">
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="49"/>
+      <c r="G2" s="32"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:61" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="48" t="s">
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="49"/>
+      <c r="G3" s="32"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:61" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -1248,165 +1248,165 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="42" t="s">
+      <c r="F4" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="43"/>
+      <c r="G4" s="34"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="44">
         <v>25</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="31"/>
-      <c r="L5" s="29">
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="46"/>
+      <c r="L5" s="44">
         <v>26</v>
       </c>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
-      <c r="P5" s="30"/>
-      <c r="Q5" s="30"/>
-      <c r="R5" s="30"/>
-      <c r="S5" s="30"/>
-      <c r="T5" s="30"/>
-      <c r="U5" s="31"/>
-      <c r="V5" s="29">
+      <c r="M5" s="45"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="45"/>
+      <c r="P5" s="45"/>
+      <c r="Q5" s="45"/>
+      <c r="R5" s="45"/>
+      <c r="S5" s="45"/>
+      <c r="T5" s="45"/>
+      <c r="U5" s="46"/>
+      <c r="V5" s="44">
         <v>27</v>
       </c>
-      <c r="W5" s="30"/>
-      <c r="X5" s="30"/>
-      <c r="Y5" s="30"/>
-      <c r="Z5" s="30"/>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="30"/>
-      <c r="AC5" s="30"/>
-      <c r="AD5" s="30"/>
-      <c r="AE5" s="31"/>
-      <c r="AF5" s="29">
+      <c r="W5" s="45"/>
+      <c r="X5" s="45"/>
+      <c r="Y5" s="45"/>
+      <c r="Z5" s="45"/>
+      <c r="AA5" s="45"/>
+      <c r="AB5" s="45"/>
+      <c r="AC5" s="45"/>
+      <c r="AD5" s="45"/>
+      <c r="AE5" s="46"/>
+      <c r="AF5" s="44">
         <v>28</v>
       </c>
-      <c r="AG5" s="30"/>
-      <c r="AH5" s="30"/>
-      <c r="AI5" s="30"/>
-      <c r="AJ5" s="30"/>
-      <c r="AK5" s="30"/>
-      <c r="AL5" s="30"/>
-      <c r="AM5" s="30"/>
-      <c r="AN5" s="30"/>
-      <c r="AO5" s="31"/>
-      <c r="AP5" s="29">
+      <c r="AG5" s="45"/>
+      <c r="AH5" s="45"/>
+      <c r="AI5" s="45"/>
+      <c r="AJ5" s="45"/>
+      <c r="AK5" s="45"/>
+      <c r="AL5" s="45"/>
+      <c r="AM5" s="45"/>
+      <c r="AN5" s="45"/>
+      <c r="AO5" s="46"/>
+      <c r="AP5" s="44">
         <v>29</v>
       </c>
-      <c r="AQ5" s="30"/>
-      <c r="AR5" s="30"/>
-      <c r="AS5" s="30"/>
-      <c r="AT5" s="30"/>
-      <c r="AU5" s="30"/>
-      <c r="AV5" s="30"/>
-      <c r="AW5" s="30"/>
-      <c r="AX5" s="30"/>
-      <c r="AY5" s="31"/>
-      <c r="AZ5" s="29">
+      <c r="AQ5" s="45"/>
+      <c r="AR5" s="45"/>
+      <c r="AS5" s="45"/>
+      <c r="AT5" s="45"/>
+      <c r="AU5" s="45"/>
+      <c r="AV5" s="45"/>
+      <c r="AW5" s="45"/>
+      <c r="AX5" s="45"/>
+      <c r="AY5" s="46"/>
+      <c r="AZ5" s="44">
         <v>30</v>
       </c>
-      <c r="BA5" s="30"/>
-      <c r="BB5" s="30"/>
-      <c r="BC5" s="30"/>
-      <c r="BD5" s="30"/>
-      <c r="BE5" s="30"/>
-      <c r="BF5" s="30"/>
-      <c r="BG5" s="30"/>
-      <c r="BH5" s="30"/>
-      <c r="BI5" s="31"/>
+      <c r="BA5" s="45"/>
+      <c r="BB5" s="45"/>
+      <c r="BC5" s="45"/>
+      <c r="BD5" s="45"/>
+      <c r="BE5" s="45"/>
+      <c r="BF5" s="45"/>
+      <c r="BG5" s="45"/>
+      <c r="BH5" s="45"/>
+      <c r="BI5" s="46"/>
     </row>
     <row r="6" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="33"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="32" t="s">
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="33"/>
-      <c r="N6" s="33"/>
-      <c r="O6" s="33"/>
-      <c r="P6" s="33"/>
-      <c r="Q6" s="33"/>
-      <c r="R6" s="33"/>
-      <c r="S6" s="33"/>
-      <c r="T6" s="33"/>
-      <c r="U6" s="34"/>
-      <c r="V6" s="32" t="s">
+      <c r="M6" s="48"/>
+      <c r="N6" s="48"/>
+      <c r="O6" s="48"/>
+      <c r="P6" s="48"/>
+      <c r="Q6" s="48"/>
+      <c r="R6" s="48"/>
+      <c r="S6" s="48"/>
+      <c r="T6" s="48"/>
+      <c r="U6" s="49"/>
+      <c r="V6" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="W6" s="33"/>
-      <c r="X6" s="33"/>
-      <c r="Y6" s="33"/>
-      <c r="Z6" s="33"/>
-      <c r="AA6" s="33"/>
-      <c r="AB6" s="33"/>
-      <c r="AC6" s="33"/>
-      <c r="AD6" s="33"/>
-      <c r="AE6" s="34"/>
-      <c r="AF6" s="32" t="s">
+      <c r="W6" s="48"/>
+      <c r="X6" s="48"/>
+      <c r="Y6" s="48"/>
+      <c r="Z6" s="48"/>
+      <c r="AA6" s="48"/>
+      <c r="AB6" s="48"/>
+      <c r="AC6" s="48"/>
+      <c r="AD6" s="48"/>
+      <c r="AE6" s="49"/>
+      <c r="AF6" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="AG6" s="33"/>
-      <c r="AH6" s="33"/>
-      <c r="AI6" s="33"/>
-      <c r="AJ6" s="33"/>
-      <c r="AK6" s="33"/>
-      <c r="AL6" s="33"/>
-      <c r="AM6" s="33"/>
-      <c r="AN6" s="33"/>
-      <c r="AO6" s="34"/>
-      <c r="AP6" s="32" t="s">
+      <c r="AG6" s="48"/>
+      <c r="AH6" s="48"/>
+      <c r="AI6" s="48"/>
+      <c r="AJ6" s="48"/>
+      <c r="AK6" s="48"/>
+      <c r="AL6" s="48"/>
+      <c r="AM6" s="48"/>
+      <c r="AN6" s="48"/>
+      <c r="AO6" s="49"/>
+      <c r="AP6" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="AQ6" s="33"/>
-      <c r="AR6" s="33"/>
-      <c r="AS6" s="33"/>
-      <c r="AT6" s="33"/>
-      <c r="AU6" s="33"/>
-      <c r="AV6" s="33"/>
-      <c r="AW6" s="33"/>
-      <c r="AX6" s="33"/>
-      <c r="AY6" s="34"/>
-      <c r="AZ6" s="32" t="s">
+      <c r="AQ6" s="48"/>
+      <c r="AR6" s="48"/>
+      <c r="AS6" s="48"/>
+      <c r="AT6" s="48"/>
+      <c r="AU6" s="48"/>
+      <c r="AV6" s="48"/>
+      <c r="AW6" s="48"/>
+      <c r="AX6" s="48"/>
+      <c r="AY6" s="49"/>
+      <c r="AZ6" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="BA6" s="33"/>
-      <c r="BB6" s="33"/>
-      <c r="BC6" s="33"/>
-      <c r="BD6" s="33"/>
-      <c r="BE6" s="33"/>
-      <c r="BF6" s="33"/>
-      <c r="BG6" s="33"/>
-      <c r="BH6" s="33"/>
-      <c r="BI6" s="34"/>
+      <c r="BA6" s="48"/>
+      <c r="BB6" s="48"/>
+      <c r="BC6" s="48"/>
+      <c r="BD6" s="48"/>
+      <c r="BE6" s="48"/>
+      <c r="BF6" s="48"/>
+      <c r="BG6" s="48"/>
+      <c r="BH6" s="48"/>
+      <c r="BI6" s="49"/>
     </row>
     <row r="7" spans="1:61" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -1597,18 +1597,18 @@
       <c r="A8" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="AZ8" s="39" t="s">
+      <c r="AZ8" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="BA8" s="40"/>
-      <c r="BB8" s="40"/>
-      <c r="BC8" s="40"/>
-      <c r="BD8" s="40"/>
-      <c r="BE8" s="40"/>
-      <c r="BF8" s="40"/>
-      <c r="BG8" s="40"/>
-      <c r="BH8" s="40"/>
-      <c r="BI8" s="41"/>
+      <c r="BA8" s="42"/>
+      <c r="BB8" s="42"/>
+      <c r="BC8" s="42"/>
+      <c r="BD8" s="42"/>
+      <c r="BE8" s="42"/>
+      <c r="BF8" s="42"/>
+      <c r="BG8" s="42"/>
+      <c r="BH8" s="42"/>
+      <c r="BI8" s="43"/>
     </row>
     <row r="9" spans="1:61" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -3012,9 +3012,9 @@
       <c r="BB30" s="7"/>
       <c r="BC30" s="10"/>
       <c r="BD30" s="10"/>
-      <c r="BE30" s="7"/>
-      <c r="BF30" s="7"/>
-      <c r="BG30" s="7"/>
+      <c r="BE30" s="10"/>
+      <c r="BF30" s="10"/>
+      <c r="BG30" s="10"/>
       <c r="BH30" s="7"/>
       <c r="BI30" s="7"/>
     </row>
@@ -3273,7 +3273,7 @@
       <c r="BI34" s="7"/>
     </row>
     <row r="35" spans="1:61" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="44" t="s">
+      <c r="A35" s="39" t="s">
         <v>40</v>
       </c>
       <c r="B35" s="5"/>
@@ -3338,7 +3338,7 @@
       <c r="BI35" s="24"/>
     </row>
     <row r="36" spans="1:61" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="45"/>
+      <c r="A36" s="40"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
@@ -5546,11 +5546,35 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="AZ6:BI6"/>
+    <mergeCell ref="L5:U5"/>
+    <mergeCell ref="V5:AE5"/>
+    <mergeCell ref="AF5:AO5"/>
+    <mergeCell ref="AP5:AY5"/>
+    <mergeCell ref="AZ5:BI5"/>
+    <mergeCell ref="B6:K6"/>
+    <mergeCell ref="L6:U6"/>
+    <mergeCell ref="V6:AE6"/>
+    <mergeCell ref="AF6:AO6"/>
+    <mergeCell ref="AP6:AY6"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="AZ8:BI8"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A61:A62"/>
     <mergeCell ref="A63:A64"/>
@@ -5567,35 +5591,11 @@
     <mergeCell ref="A33:A34"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="AZ8:BI8"/>
-    <mergeCell ref="B5:K5"/>
-    <mergeCell ref="AZ6:BI6"/>
-    <mergeCell ref="L5:U5"/>
-    <mergeCell ref="V5:AE5"/>
-    <mergeCell ref="AF5:AO5"/>
-    <mergeCell ref="AP5:AY5"/>
-    <mergeCell ref="AZ5:BI5"/>
-    <mergeCell ref="B6:K6"/>
-    <mergeCell ref="L6:U6"/>
-    <mergeCell ref="V6:AE6"/>
-    <mergeCell ref="AF6:AO6"/>
-    <mergeCell ref="AP6:AY6"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5615,12 +5615,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="47"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30"/>
       <c r="F1" s="18" t="s">
         <v>8</v>
       </c>
@@ -5639,29 +5639,29 @@
       <c r="Q1" s="17"/>
     </row>
     <row r="2" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="48" t="s">
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="49"/>
+      <c r="G2" s="32"/>
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:52" ht="21" x14ac:dyDescent="0.4">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="48" t="s">
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="49"/>
+      <c r="G3" s="32"/>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:52" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -5669,222 +5669,222 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
-      <c r="F4" s="42" t="s">
+      <c r="F4" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="43"/>
+      <c r="G4" s="34"/>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="44">
         <v>8</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="29">
+      <c r="C5" s="45"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="44">
         <v>9</v>
       </c>
-      <c r="F5" s="30"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="50" t="s">
+      <c r="F5" s="45"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="51"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="29">
+      <c r="I5" s="54"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="44">
         <v>11</v>
       </c>
-      <c r="L5" s="30"/>
-      <c r="M5" s="31"/>
-      <c r="N5" s="50" t="s">
+      <c r="L5" s="45"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="51"/>
-      <c r="P5" s="52"/>
-      <c r="Q5" s="29">
+      <c r="O5" s="54"/>
+      <c r="P5" s="55"/>
+      <c r="Q5" s="44">
         <v>13</v>
       </c>
-      <c r="R5" s="30"/>
-      <c r="S5" s="31"/>
-      <c r="T5" s="29">
+      <c r="R5" s="45"/>
+      <c r="S5" s="46"/>
+      <c r="T5" s="44">
         <v>14</v>
       </c>
-      <c r="U5" s="30"/>
-      <c r="V5" s="31"/>
-      <c r="W5" s="59">
+      <c r="U5" s="45"/>
+      <c r="V5" s="46"/>
+      <c r="W5" s="56">
         <v>15</v>
       </c>
-      <c r="X5" s="60"/>
-      <c r="Y5" s="61"/>
-      <c r="Z5" s="29">
+      <c r="X5" s="57"/>
+      <c r="Y5" s="58"/>
+      <c r="Z5" s="44">
         <v>16</v>
       </c>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="31"/>
-      <c r="AC5" s="29">
+      <c r="AA5" s="45"/>
+      <c r="AB5" s="46"/>
+      <c r="AC5" s="44">
         <v>17</v>
       </c>
-      <c r="AD5" s="30"/>
-      <c r="AE5" s="31"/>
-      <c r="AF5" s="29">
+      <c r="AD5" s="45"/>
+      <c r="AE5" s="46"/>
+      <c r="AF5" s="44">
         <v>18</v>
       </c>
-      <c r="AG5" s="30"/>
-      <c r="AH5" s="31"/>
-      <c r="AI5" s="29">
+      <c r="AG5" s="45"/>
+      <c r="AH5" s="46"/>
+      <c r="AI5" s="44">
         <v>19</v>
       </c>
-      <c r="AJ5" s="30"/>
-      <c r="AK5" s="31"/>
-      <c r="AL5" s="29">
+      <c r="AJ5" s="45"/>
+      <c r="AK5" s="46"/>
+      <c r="AL5" s="44">
         <v>20</v>
       </c>
-      <c r="AM5" s="30"/>
-      <c r="AN5" s="31"/>
-      <c r="AO5" s="29">
+      <c r="AM5" s="45"/>
+      <c r="AN5" s="46"/>
+      <c r="AO5" s="44">
         <v>21</v>
       </c>
-      <c r="AP5" s="30"/>
-      <c r="AQ5" s="31"/>
-      <c r="AR5" s="29">
+      <c r="AP5" s="45"/>
+      <c r="AQ5" s="46"/>
+      <c r="AR5" s="44">
         <v>22</v>
       </c>
-      <c r="AS5" s="30"/>
-      <c r="AT5" s="31"/>
-      <c r="AU5" s="29">
+      <c r="AS5" s="45"/>
+      <c r="AT5" s="46"/>
+      <c r="AU5" s="44">
         <v>23</v>
       </c>
-      <c r="AV5" s="30"/>
-      <c r="AW5" s="31"/>
-      <c r="AX5" s="50">
+      <c r="AV5" s="45"/>
+      <c r="AW5" s="46"/>
+      <c r="AX5" s="53">
         <v>24</v>
       </c>
-      <c r="AY5" s="51"/>
-      <c r="AZ5" s="52"/>
+      <c r="AY5" s="54"/>
+      <c r="AZ5" s="55"/>
     </row>
     <row r="6" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="47">
         <v>16.02</v>
       </c>
-      <c r="C6" s="34"/>
+      <c r="C6" s="49"/>
       <c r="D6" s="2">
         <v>19.02</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="47">
         <v>23.02</v>
       </c>
-      <c r="F6" s="34"/>
+      <c r="F6" s="49"/>
       <c r="G6" s="2">
         <v>26.02</v>
       </c>
-      <c r="H6" s="32">
+      <c r="H6" s="47">
         <v>2.0299999999999998</v>
       </c>
-      <c r="I6" s="34"/>
+      <c r="I6" s="49"/>
       <c r="J6" s="2">
         <v>5.03</v>
       </c>
-      <c r="K6" s="32">
+      <c r="K6" s="47">
         <v>9.0299999999999994</v>
       </c>
-      <c r="L6" s="34"/>
+      <c r="L6" s="49"/>
       <c r="M6" s="2">
         <v>12.03</v>
       </c>
-      <c r="N6" s="32">
+      <c r="N6" s="47">
         <v>16.03</v>
       </c>
-      <c r="O6" s="34"/>
+      <c r="O6" s="49"/>
       <c r="P6" s="2">
         <v>19.03</v>
       </c>
-      <c r="Q6" s="32">
+      <c r="Q6" s="47">
         <v>23.03</v>
       </c>
-      <c r="R6" s="34"/>
+      <c r="R6" s="49"/>
       <c r="S6" s="2">
         <v>26.03</v>
       </c>
-      <c r="T6" s="32">
+      <c r="T6" s="47">
         <v>30.03</v>
       </c>
-      <c r="U6" s="34"/>
+      <c r="U6" s="49"/>
       <c r="V6" s="2">
         <v>2.04</v>
       </c>
-      <c r="W6" s="62">
+      <c r="W6" s="59">
         <v>6.04</v>
       </c>
-      <c r="X6" s="63"/>
+      <c r="X6" s="60"/>
       <c r="Y6" s="3">
         <v>9.0399999999999991</v>
       </c>
-      <c r="Z6" s="32">
+      <c r="Z6" s="47">
         <v>13.04</v>
       </c>
-      <c r="AA6" s="34"/>
+      <c r="AA6" s="49"/>
       <c r="AB6" s="2">
         <v>16.04</v>
       </c>
-      <c r="AC6" s="32">
+      <c r="AC6" s="47">
         <v>20.04</v>
       </c>
-      <c r="AD6" s="34"/>
+      <c r="AD6" s="49"/>
       <c r="AE6" s="2">
         <v>23.04</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="47">
         <v>27.04</v>
       </c>
-      <c r="AG6" s="34"/>
+      <c r="AG6" s="49"/>
       <c r="AH6" s="2">
         <v>30.04</v>
       </c>
-      <c r="AI6" s="32">
+      <c r="AI6" s="47">
         <v>4.05</v>
       </c>
-      <c r="AJ6" s="34"/>
+      <c r="AJ6" s="49"/>
       <c r="AK6" s="2">
         <v>7.05</v>
       </c>
-      <c r="AL6" s="32">
+      <c r="AL6" s="47">
         <v>11.05</v>
       </c>
-      <c r="AM6" s="34"/>
+      <c r="AM6" s="49"/>
       <c r="AN6" s="2">
         <v>14.05</v>
       </c>
-      <c r="AO6" s="32">
+      <c r="AO6" s="47">
         <v>18.05</v>
       </c>
-      <c r="AP6" s="34"/>
+      <c r="AP6" s="49"/>
       <c r="AQ6" s="2">
         <v>21.05</v>
       </c>
-      <c r="AR6" s="32">
+      <c r="AR6" s="47">
         <v>25.05</v>
       </c>
-      <c r="AS6" s="34"/>
+      <c r="AS6" s="49"/>
       <c r="AT6" s="2">
         <v>28.05</v>
       </c>
-      <c r="AU6" s="32">
+      <c r="AU6" s="47">
         <v>1.06</v>
       </c>
-      <c r="AV6" s="34"/>
+      <c r="AV6" s="49"/>
       <c r="AW6" s="2">
         <v>4.0599999999999996</v>
       </c>
-      <c r="AX6" s="32">
+      <c r="AX6" s="47">
         <v>8.06</v>
       </c>
-      <c r="AY6" s="34"/>
+      <c r="AY6" s="49"/>
       <c r="AZ6" s="2">
         <v>11.06</v>
       </c>
@@ -6051,32 +6051,32 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="39" t="s">
+      <c r="H8" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="40"/>
-      <c r="J8" s="41"/>
-      <c r="K8" s="64" t="s">
+      <c r="I8" s="42"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="61" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="65"/>
-      <c r="M8" s="66"/>
-      <c r="N8" s="53" t="s">
+      <c r="L8" s="62"/>
+      <c r="M8" s="63"/>
+      <c r="N8" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="O8" s="54"/>
-      <c r="P8" s="55"/>
+      <c r="O8" s="65"/>
+      <c r="P8" s="66"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
-      <c r="W8" s="56" t="s">
+      <c r="W8" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="X8" s="57"/>
-      <c r="Y8" s="58"/>
+      <c r="X8" s="51"/>
+      <c r="Y8" s="52"/>
       <c r="Z8" s="4"/>
       <c r="AA8" s="4"/>
       <c r="AB8" s="4"/>
@@ -6101,11 +6101,11 @@
       <c r="AU8" s="4"/>
       <c r="AV8" s="4"/>
       <c r="AW8" s="4"/>
-      <c r="AX8" s="39" t="s">
+      <c r="AX8" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="AY8" s="40"/>
-      <c r="AZ8" s="41"/>
+      <c r="AY8" s="42"/>
+      <c r="AZ8" s="43"/>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
@@ -7976,7 +7976,7 @@
       <c r="AZ42" s="7"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A43" s="44" t="s">
+      <c r="A43" s="39" t="s">
         <v>40</v>
       </c>
       <c r="B43" s="5"/>
@@ -8032,7 +8032,7 @@
       <c r="AZ43" s="5"/>
     </row>
     <row r="44" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="45"/>
+      <c r="A44" s="40"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -8197,6 +8197,54 @@
     </row>
   </sheetData>
   <mergeCells count="64">
+    <mergeCell ref="AU5:AW5"/>
+    <mergeCell ref="AU6:AV6"/>
+    <mergeCell ref="AX5:AZ5"/>
+    <mergeCell ref="AX6:AY6"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="AO6:AP6"/>
+    <mergeCell ref="AR5:AT5"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="AC6:AD6"/>
+    <mergeCell ref="AF5:AH5"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H6:I6"/>
     <mergeCell ref="AX8:AZ8"/>
     <mergeCell ref="W8:Y8"/>
     <mergeCell ref="K5:M5"/>
@@ -8213,54 +8261,6 @@
     <mergeCell ref="Z6:AA6"/>
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="AC5:AE5"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="AC6:AD6"/>
-    <mergeCell ref="AF5:AH5"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="AU5:AW5"/>
-    <mergeCell ref="AU6:AV6"/>
-    <mergeCell ref="AX5:AZ5"/>
-    <mergeCell ref="AX6:AY6"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="AL6:AM6"/>
-    <mergeCell ref="AO5:AQ5"/>
-    <mergeCell ref="AO6:AP6"/>
-    <mergeCell ref="AR5:AT5"/>
-    <mergeCell ref="AR6:AS6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>